<commit_message>
feat(deploy): enable 1-click free GitHub Pages and Static deployment with zero credit card
</commit_message>
<xml_diff>
--- a/data/aiesec_egypt_events_latest.xlsx
+++ b/data/aiesec_egypt_events_latest.xlsx
@@ -21005,12 +21005,12 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
+          <t>Cairo University Engineering Annual Employment Fair &amp; Tech Conclave</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Sep 20, 2026 · 09:00 AM</t>
+          <t>Sep 24, 2026 · 09:30 AM</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -21020,17 +21020,17 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
+          <t>Cairo University Faculty of Engineering, Grand Celebration Hall &amp; Outdoor Engineering Quad (Building 2)</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Technology &amp; Hackathons</t>
+          <t>Career Fair &amp; Employment</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -21040,7 +21040,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>Free Team Registration / Competitive Selection</t>
+          <t>Free Student Admission (Valid University ID Required)</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -21060,7 +21060,7 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>student, university, campus, cairo university, hackathon, developer</t>
+          <t>employment, internship, cv, student, university, undergraduate</t>
         </is>
       </c>
       <c r="M277" t="inlineStr">
@@ -21070,29 +21070,29 @@
       </c>
       <c r="N277" t="inlineStr">
         <is>
-          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
+          <t>Cairo University Faculty of Engineering Student Union</t>
         </is>
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>https://t.me/s/egypt_tech_events</t>
+          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
         </is>
       </c>
       <c r="P277" t="inlineStr">
         <is>
-          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
+          <t>The premier university employment gathering for engineering and computer science students in Egypt. Attracts 50+ multinational software houses, civil engineering contractors, and energy conglomerates. Features 16 technical panel sessions, live 1-on-1 CV screening clinics, and walk-in interviews. Target Audience: Undergraduates and fresh alumni from Computer, Communications, Mechanical, Civil, and Architectural Engineering. Venue Details: Grand Celebration Hall (Building 2, Ground Floor) &amp; Outdoor Plaza, Giza. Expected Footfall: 4,000+ attendees over 2 days. Entry is free upon presenting an active university ID. AIESEC Tactical Opportunity: High-yield activation zone for Global Talent (GT) technical internship sales and direct recruiting of high-achieving student leaders.</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
+          <t>Ain Shams University Youth Innovation &amp; Student Leadership Symposium</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Sep 25, 2026 · 06:00 PM</t>
+          <t>Sep 30, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -21102,12 +21102,12 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
+          <t>Ain Shams University Al-Zaafaran Palace Conference Hall &amp; Main Campus Complex, Abbassia</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -21122,7 +21122,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>Free Open Broadcast &amp; Webinar Series</t>
+          <t>Free Entry / Online Pre-Registration</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -21142,7 +21142,7 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>student, university, campus, youth, leadership, volunteer</t>
+          <t>recruitment, student, university, campus, youth, ain shams</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
@@ -21152,29 +21152,29 @@
       </c>
       <c r="N278" t="inlineStr">
         <is>
-          <t>Telegram Channel @student_opportunities_eg</t>
+          <t>Ain Shams University Central Student Union</t>
         </is>
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>https://t.me/s/student_opportunities_eg</t>
+          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
         </is>
       </c>
       <c r="P278" t="inlineStr">
         <is>
-          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
+          <t>Comprehensive 2-day student union symposium convening student leaders and active youth across 16 faculties. Program highlights include a campus social entrepreneurship pitch competition with 250,000 EGP in incubation vouchers, 8 interactive roundtables on youth civil engagement, and cross-cultural communication masterclasses. Target Audience: Students across Business/Commerce, Computer Science, Engineering, Medicine, and Languages (Al-Alsun). Venue Details: Al-Zaafaran Historical Palace Conference Hall &amp; Stadium Courtyard, Abbassia, Cairo. Expected Scale: 3,500+ attendees. Open admission with digital registration pass. AIESEC Tactical Opportunity: Prime talent pipeline for Global Volunteer (GV) social impact exchanges and Local Committee member recruitment.</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
+          <t>Tanta University Science, Pharmacy &amp; Tech Innovation Expo</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Sep 29, 2026 · 05:00 PM</t>
+          <t>Oct 04, 2026 · 10:30 AM</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -21184,12 +21184,12 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
+          <t>Tanta University Complex (Sebor Medical &amp; Science Quad), Hall 3 &amp; Open Courtyard, El-Gharbia</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -21204,7 +21204,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
+          <t>Free Student Entry (National / Student ID)</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -21224,7 +21224,7 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>internship, student, university, undergraduate, web development, leadership</t>
+          <t>career, student, university, undergraduate, software, volunteer</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
@@ -21234,39 +21234,39 @@
       </c>
       <c r="N279" t="inlineStr">
         <is>
-          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
+          <t>Tanta University Student Union &amp; Faculty of Science</t>
         </is>
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>https://t.me/s/delta_youth_events</t>
+          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
         </is>
       </c>
       <c r="P279" t="inlineStr">
         <is>
-          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
+          <t>The central student innovation showcase for the Gharbia and Middle Delta governorates. Features 30+ university scientific exhibits, biotechnology research posters, pharmaceutical career tracks, and regional software development showcases. Target Audience: Undergraduates and recent graduates from Faculties of Science, Pharmacy, Medicine, and Information Technology across Tanta, Kafr El-Sheikh, and Menoufia. Venue Details: Tanta University Complex (Sebor), Hall 3 and Central Exhibition Courtyard, Tanta. Expected Scale: 2,200+ students. Free admission with valid student or national ID. AIESEC Tactical Opportunity: ABSOLUTE HOME TURF PRIORITY for AIESEC in Tanta: Maximum brand presence, Global Volunteer sign-ups, and executive networking with faculty deans.</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Cairo University Engineering Annual Employment Fair &amp; Tech Conclave</t>
+          <t>Alexandria University Youth Empowerment &amp; Entrepreneurship Summit</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Sep 24, 2026 · 09:30 AM</t>
+          <t>Sep 27, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Alexandria</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Cairo University Faculty of Engineering, Grand Celebration Hall &amp; Outdoor Engineering Quad (Building 2)</t>
+          <t>Alexandria University Faculty of Commerce Main Auditorium &amp; Maritime Courtyard, Shatby</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -21286,7 +21286,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>Free Student Admission (Valid University ID Required)</t>
+          <t>Free Registration via Campus Link</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -21306,7 +21306,7 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>employment, internship, cv, student, university, undergraduate</t>
+          <t>internship, resume, student, university, campus, youth</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
@@ -21316,39 +21316,39 @@
       </c>
       <c r="N280" t="inlineStr">
         <is>
-          <t>Cairo University Faculty of Engineering Student Union</t>
+          <t>Alexandria University Student Activity Council</t>
         </is>
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
+          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
         </is>
       </c>
       <c r="P280" t="inlineStr">
         <is>
-          <t>The premier university employment gathering for engineering and computer science students in Egypt. Attracts 50+ multinational software houses, civil engineering contractors, and energy conglomerates. Features 16 technical panel sessions, live 1-on-1 CV screening clinics, and walk-in interviews. Target Audience: Undergraduates and fresh alumni from Computer, Communications, Mechanical, Civil, and Architectural Engineering. Venue Details: Grand Celebration Hall (Building 2, Ground Floor) &amp; Outdoor Plaza, Giza. Expected Footfall: 4,000+ attendees over 2 days. Entry is free upon presenting an active university ID. AIESEC Tactical Opportunity: High-yield activation zone for Global Talent (GT) technical internship sales and direct recruiting of high-achieving student leaders.</t>
+          <t>Alexandria's foremost campus entrepreneurship day bringing together commercial leaders, startup founders, and university talent. Agenda includes corporate panels on North Coast maritime logistics, fintech development, digital marketing trends, and resume critique clinics with senior HR specialists. Target Audience: Commerce, Business Information Systems (BIS), Economics, Arts, and Engineering students. Venue Details: Faculty of Commerce Main Auditorium and Maritime Courtyard, Shatby, Alexandria. Expected Scale: 2,500+ undergraduate delegates. Free admission with pre-issued QR code. AIESEC Tactical Opportunity: Joint activation potential for LC Tanta and LC Alexandria to drive Global Talent business internship applications.</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Ain Shams University Youth Innovation &amp; Student Leadership Symposium</t>
+          <t>Mansoura University Annual Career &amp; Coding Conclave</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Sep 30, 2026 · 10:00 AM</t>
+          <t>Oct 11, 2026 · 09:00 AM</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Mansoura</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Ain Shams University Al-Zaafaran Palace Conference Hall &amp; Main Campus Complex, Abbassia</t>
+          <t>Mansoura University Convention Centre &amp; Faculty of Computers Grounds, Dakahlia</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -21358,7 +21358,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>Youth Leadership &amp; Student Orgs</t>
+          <t>Technology &amp; Hackathons</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
@@ -21368,7 +21368,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>Free Entry / Online Pre-Registration</t>
+          <t>Free Student Entry</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -21388,54 +21388,54 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>recruitment, student, university, campus, youth, ain shams</t>
+          <t>career, recruitment, student, university, coding, software</t>
         </is>
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+          <t>Promote Global Talent IT &amp; Tech Internship Opportunities</t>
         </is>
       </c>
       <c r="N281" t="inlineStr">
         <is>
-          <t>Ain Shams University Central Student Union</t>
+          <t>Mansoura University Faculty of Computers &amp; Artificial Intelligence</t>
         </is>
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
+          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
         </is>
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>Comprehensive 2-day student union symposium convening student leaders and active youth across 16 faculties. Program highlights include a campus social entrepreneurship pitch competition with 250,000 EGP in incubation vouchers, 8 interactive roundtables on youth civil engagement, and cross-cultural communication masterclasses. Target Audience: Students across Business/Commerce, Computer Science, Engineering, Medicine, and Languages (Al-Alsun). Venue Details: Al-Zaafaran Historical Palace Conference Hall &amp; Stadium Courtyard, Abbassia, Cairo. Expected Scale: 3,500+ attendees. Open admission with digital registration pass. AIESEC Tactical Opportunity: Prime talent pipeline for Global Volunteer (GV) social impact exchanges and Local Committee member recruitment.</t>
+          <t>The East Delta's flagship computer science and software engineering conference. Features 20+ recruiting technology firms, a 12-hour algorithmic problem-solving sprint, workshops on Generative AI and Cybersecurity, and technical mock interviews. Target Audience: Students and alumni from Computers &amp; Artificial Intelligence, Engineering, and Mathematics across Mansoura and Damietta. Venue Details: Mansoura University Main Convention Centre, Jihan Street, Mansoura. Expected Scale: 1,800+ aspiring software engineers. Free admission with student credential. AIESEC Tactical Opportunity: High-value recruitment ground for AIESEC Global Talent tech placements abroad.</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Tanta University Science, Pharmacy &amp; Tech Innovation Expo</t>
+          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Oct 04, 2026 · 10:30 AM</t>
+          <t>Sep 20, 2026 · 09:00 AM</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Tanta University Complex (Sebor Medical &amp; Science Quad), Hall 3 &amp; Open Courtyard, El-Gharbia</t>
+          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -21450,7 +21450,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>Free Student Entry (National / Student ID)</t>
+          <t>Free Team Registration / Competitive Selection</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -21470,7 +21470,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>career, student, university, undergraduate, software, volunteer</t>
+          <t>student, university, campus, cairo university, hackathon, developer</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
@@ -21480,49 +21480,49 @@
       </c>
       <c r="N282" t="inlineStr">
         <is>
-          <t>Tanta University Student Union &amp; Faculty of Science</t>
+          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
         </is>
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
+          <t>https://t.me/s/egypt_tech_events</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>The central student innovation showcase for the Gharbia and Middle Delta governorates. Features 30+ university scientific exhibits, biotechnology research posters, pharmaceutical career tracks, and regional software development showcases. Target Audience: Undergraduates and recent graduates from Faculties of Science, Pharmacy, Medicine, and Information Technology across Tanta, Kafr El-Sheikh, and Menoufia. Venue Details: Tanta University Complex (Sebor), Hall 3 and Central Exhibition Courtyard, Tanta. Expected Scale: 2,200+ students. Free admission with valid student or national ID. AIESEC Tactical Opportunity: ABSOLUTE HOME TURF PRIORITY for AIESEC in Tanta: Maximum brand presence, Global Volunteer sign-ups, and executive networking with faculty deans.</t>
+          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Alexandria University Youth Empowerment &amp; Entrepreneurship Summit</t>
+          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Sep 27, 2026 · 10:00 AM</t>
+          <t>Sep 25, 2026 · 06:00 PM</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Alexandria</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Alexandria University Faculty of Commerce Main Auditorium &amp; Maritime Courtyard, Shatby</t>
+          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Career Fair &amp; Employment</t>
+          <t>Youth Leadership &amp; Student Orgs</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
@@ -21532,7 +21532,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>Free Registration via Campus Link</t>
+          <t>Free Open Broadcast &amp; Webinar Series</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -21552,7 +21552,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>internship, resume, student, university, campus, youth</t>
+          <t>student, university, campus, youth, leadership, volunteer</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
@@ -21562,44 +21562,44 @@
       </c>
       <c r="N283" t="inlineStr">
         <is>
-          <t>Alexandria University Student Activity Council</t>
+          <t>Telegram Channel @student_opportunities_eg</t>
         </is>
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
+          <t>https://t.me/s/student_opportunities_eg</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
         <is>
-          <t>Alexandria's foremost campus entrepreneurship day bringing together commercial leaders, startup founders, and university talent. Agenda includes corporate panels on North Coast maritime logistics, fintech development, digital marketing trends, and resume critique clinics with senior HR specialists. Target Audience: Commerce, Business Information Systems (BIS), Economics, Arts, and Engineering students. Venue Details: Faculty of Commerce Main Auditorium and Maritime Courtyard, Shatby, Alexandria. Expected Scale: 2,500+ undergraduate delegates. Free admission with pre-issued QR code. AIESEC Tactical Opportunity: Joint activation potential for LC Tanta and LC Alexandria to drive Global Talent business internship applications.</t>
+          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Mansoura University Annual Career &amp; Coding Conclave</t>
+          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Oct 11, 2026 · 09:00 AM</t>
+          <t>Sep 29, 2026 · 05:00 PM</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Mansoura</t>
+          <t>Tanta</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Mansoura University Convention Centre &amp; Faculty of Computers Grounds, Dakahlia</t>
+          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -21614,7 +21614,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>Free Student Entry</t>
+          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -21634,27 +21634,27 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>career, recruitment, student, university, coding, software</t>
+          <t>internship, student, university, undergraduate, web development, leadership</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>Promote Global Talent IT &amp; Tech Internship Opportunities</t>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
         </is>
       </c>
       <c r="N284" t="inlineStr">
         <is>
-          <t>Mansoura University Faculty of Computers &amp; Artificial Intelligence</t>
+          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
         </is>
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
+          <t>https://t.me/s/delta_youth_events</t>
         </is>
       </c>
       <c r="P284" t="inlineStr">
         <is>
-          <t>The East Delta's flagship computer science and software engineering conference. Features 20+ recruiting technology firms, a 12-hour algorithmic problem-solving sprint, workshops on Generative AI and Cybersecurity, and technical mock interviews. Target Audience: Students and alumni from Computers &amp; Artificial Intelligence, Engineering, and Mathematics across Mansoura and Damietta. Venue Details: Mansoura University Main Convention Centre, Jihan Street, Mansoura. Expected Scale: 1,800+ aspiring software engineers. Free admission with student credential. AIESEC Tactical Opportunity: High-value recruitment ground for AIESEC Global Talent tech placements abroad.</t>
+          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement 3D holographic card tilt with iridescent sheen (1) and interactive mouse-repellent cosmic dust particles (6)
</commit_message>
<xml_diff>
--- a/data/aiesec_egypt_events_latest.xlsx
+++ b/data/aiesec_egypt_events_latest.xlsx
@@ -24014,12 +24014,12 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
+          <t>Cairo University Engineering Annual Employment Fair &amp; Tech Conclave</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Sep 20, 2026 · 09:00 AM</t>
+          <t>Sep 24, 2026 · 09:30 AM</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -24029,17 +24029,17 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
+          <t>Cairo University Faculty of Engineering, Grand Celebration Hall &amp; Outdoor Engineering Quad (Building 2)</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>Technology &amp; Hackathons</t>
+          <t>Career Fair &amp; Employment</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
@@ -24049,7 +24049,7 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>Free Team Registration / Competitive Selection</t>
+          <t>Free Student Admission (Valid University ID Required)</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -24069,7 +24069,7 @@
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t>student, university, campus, cairo university, hackathon, developer</t>
+          <t>employment, internship, cv, student, university, undergraduate</t>
         </is>
       </c>
       <c r="M312" t="inlineStr">
@@ -24079,29 +24079,29 @@
       </c>
       <c r="N312" t="inlineStr">
         <is>
-          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
+          <t>Cairo University Faculty of Engineering Student Union</t>
         </is>
       </c>
       <c r="O312" t="inlineStr">
         <is>
-          <t>https://t.me/s/egypt_tech_events</t>
+          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
         </is>
       </c>
       <c r="P312" t="inlineStr">
         <is>
-          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
+          <t>The premier university employment gathering for engineering and computer science students in Egypt. Attracts 50+ multinational software houses, civil engineering contractors, and energy conglomerates. Features 16 technical panel sessions, live 1-on-1 CV screening clinics, and walk-in interviews. Target Audience: Undergraduates and fresh alumni from Computer, Communications, Mechanical, Civil, and Architectural Engineering. Venue Details: Grand Celebration Hall (Building 2, Ground Floor) &amp; Outdoor Plaza, Giza. Expected Footfall: 4,000+ attendees over 2 days. Entry is free upon presenting an active university ID. AIESEC Tactical Opportunity: High-yield activation zone for Global Talent (GT) technical internship sales and direct recruiting of high-achieving student leaders.</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
+          <t>Ain Shams University Youth Innovation &amp; Student Leadership Symposium</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Sep 25, 2026 · 06:00 PM</t>
+          <t>Sep 30, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -24111,12 +24111,12 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
+          <t>Ain Shams University Al-Zaafaran Palace Conference Hall &amp; Main Campus Complex, Abbassia</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
@@ -24131,7 +24131,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>Free Open Broadcast &amp; Webinar Series</t>
+          <t>Free Entry / Online Pre-Registration</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -24151,7 +24151,7 @@
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t>student, university, campus, youth, leadership, volunteer</t>
+          <t>recruitment, student, university, campus, youth, ain shams</t>
         </is>
       </c>
       <c r="M313" t="inlineStr">
@@ -24161,29 +24161,29 @@
       </c>
       <c r="N313" t="inlineStr">
         <is>
-          <t>Telegram Channel @student_opportunities_eg</t>
+          <t>Ain Shams University Central Student Union</t>
         </is>
       </c>
       <c r="O313" t="inlineStr">
         <is>
-          <t>https://t.me/s/student_opportunities_eg</t>
+          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
         </is>
       </c>
       <c r="P313" t="inlineStr">
         <is>
-          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
+          <t>Comprehensive 2-day student union symposium convening student leaders and active youth across 16 faculties. Program highlights include a campus social entrepreneurship pitch competition with 250,000 EGP in incubation vouchers, 8 interactive roundtables on youth civil engagement, and cross-cultural communication masterclasses. Target Audience: Students across Business/Commerce, Computer Science, Engineering, Medicine, and Languages (Al-Alsun). Venue Details: Al-Zaafaran Historical Palace Conference Hall &amp; Stadium Courtyard, Abbassia, Cairo. Expected Scale: 3,500+ attendees. Open admission with digital registration pass. AIESEC Tactical Opportunity: Prime talent pipeline for Global Volunteer (GV) social impact exchanges and Local Committee member recruitment.</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
+          <t>Tanta University Science, Pharmacy &amp; Tech Innovation Expo</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Sep 29, 2026 · 05:00 PM</t>
+          <t>Oct 04, 2026 · 10:30 AM</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -24193,12 +24193,12 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
+          <t>Tanta University Complex (Sebor Medical &amp; Science Quad), Hall 3 &amp; Open Courtyard, El-Gharbia</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -24213,7 +24213,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
+          <t>Free Student Entry (National / Student ID)</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
@@ -24233,7 +24233,7 @@
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>internship, student, university, undergraduate, web development, leadership</t>
+          <t>career, student, university, undergraduate, software, volunteer</t>
         </is>
       </c>
       <c r="M314" t="inlineStr">
@@ -24243,39 +24243,39 @@
       </c>
       <c r="N314" t="inlineStr">
         <is>
-          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
+          <t>Tanta University Student Union &amp; Faculty of Science</t>
         </is>
       </c>
       <c r="O314" t="inlineStr">
         <is>
-          <t>https://t.me/s/delta_youth_events</t>
+          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
         </is>
       </c>
       <c r="P314" t="inlineStr">
         <is>
-          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
+          <t>The central student innovation showcase for the Gharbia and Middle Delta governorates. Features 30+ university scientific exhibits, biotechnology research posters, pharmaceutical career tracks, and regional software development showcases. Target Audience: Undergraduates and recent graduates from Faculties of Science, Pharmacy, Medicine, and Information Technology across Tanta, Kafr El-Sheikh, and Menoufia. Venue Details: Tanta University Complex (Sebor), Hall 3 and Central Exhibition Courtyard, Tanta. Expected Scale: 2,200+ students. Free admission with valid student or national ID. AIESEC Tactical Opportunity: ABSOLUTE HOME TURF PRIORITY for AIESEC in Tanta: Maximum brand presence, Global Volunteer sign-ups, and executive networking with faculty deans.</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Cairo University Engineering Annual Employment Fair &amp; Tech Conclave</t>
+          <t>Alexandria University Youth Empowerment &amp; Entrepreneurship Summit</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Sep 24, 2026 · 09:30 AM</t>
+          <t>Sep 27, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Alexandria</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Cairo University Faculty of Engineering, Grand Celebration Hall &amp; Outdoor Engineering Quad (Building 2)</t>
+          <t>Alexandria University Faculty of Commerce Main Auditorium &amp; Maritime Courtyard, Shatby</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -24295,7 +24295,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>Free Student Admission (Valid University ID Required)</t>
+          <t>Free Registration via Campus Link</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="L315" t="inlineStr">
         <is>
-          <t>employment, internship, cv, student, university, undergraduate</t>
+          <t>internship, resume, student, university, campus, youth</t>
         </is>
       </c>
       <c r="M315" t="inlineStr">
@@ -24325,39 +24325,39 @@
       </c>
       <c r="N315" t="inlineStr">
         <is>
-          <t>Cairo University Faculty of Engineering Student Union</t>
+          <t>Alexandria University Student Activity Council</t>
         </is>
       </c>
       <c r="O315" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
+          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
         </is>
       </c>
       <c r="P315" t="inlineStr">
         <is>
-          <t>The premier university employment gathering for engineering and computer science students in Egypt. Attracts 50+ multinational software houses, civil engineering contractors, and energy conglomerates. Features 16 technical panel sessions, live 1-on-1 CV screening clinics, and walk-in interviews. Target Audience: Undergraduates and fresh alumni from Computer, Communications, Mechanical, Civil, and Architectural Engineering. Venue Details: Grand Celebration Hall (Building 2, Ground Floor) &amp; Outdoor Plaza, Giza. Expected Footfall: 4,000+ attendees over 2 days. Entry is free upon presenting an active university ID. AIESEC Tactical Opportunity: High-yield activation zone for Global Talent (GT) technical internship sales and direct recruiting of high-achieving student leaders.</t>
+          <t>Alexandria's foremost campus entrepreneurship day bringing together commercial leaders, startup founders, and university talent. Agenda includes corporate panels on North Coast maritime logistics, fintech development, digital marketing trends, and resume critique clinics with senior HR specialists. Target Audience: Commerce, Business Information Systems (BIS), Economics, Arts, and Engineering students. Venue Details: Faculty of Commerce Main Auditorium and Maritime Courtyard, Shatby, Alexandria. Expected Scale: 2,500+ undergraduate delegates. Free admission with pre-issued QR code. AIESEC Tactical Opportunity: Joint activation potential for LC Tanta and LC Alexandria to drive Global Talent business internship applications.</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Ain Shams University Youth Innovation &amp; Student Leadership Symposium</t>
+          <t>Mansoura University Annual Career &amp; Coding Conclave</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Sep 30, 2026 · 10:00 AM</t>
+          <t>Oct 11, 2026 · 09:00 AM</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Mansoura</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Ain Shams University Al-Zaafaran Palace Conference Hall &amp; Main Campus Complex, Abbassia</t>
+          <t>Mansoura University Convention Centre &amp; Faculty of Computers Grounds, Dakahlia</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -24367,7 +24367,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>Youth Leadership &amp; Student Orgs</t>
+          <t>Technology &amp; Hackathons</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
@@ -24377,7 +24377,7 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>Free Entry / Online Pre-Registration</t>
+          <t>Free Student Entry</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
@@ -24397,54 +24397,54 @@
       </c>
       <c r="L316" t="inlineStr">
         <is>
-          <t>recruitment, student, university, campus, youth, ain shams</t>
+          <t>career, recruitment, student, university, coding, software</t>
         </is>
       </c>
       <c r="M316" t="inlineStr">
         <is>
-          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+          <t>Promote Global Talent IT &amp; Tech Internship Opportunities</t>
         </is>
       </c>
       <c r="N316" t="inlineStr">
         <is>
-          <t>Ain Shams University Central Student Union</t>
+          <t>Mansoura University Faculty of Computers &amp; Artificial Intelligence</t>
         </is>
       </c>
       <c r="O316" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
+          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
         </is>
       </c>
       <c r="P316" t="inlineStr">
         <is>
-          <t>Comprehensive 2-day student union symposium convening student leaders and active youth across 16 faculties. Program highlights include a campus social entrepreneurship pitch competition with 250,000 EGP in incubation vouchers, 8 interactive roundtables on youth civil engagement, and cross-cultural communication masterclasses. Target Audience: Students across Business/Commerce, Computer Science, Engineering, Medicine, and Languages (Al-Alsun). Venue Details: Al-Zaafaran Historical Palace Conference Hall &amp; Stadium Courtyard, Abbassia, Cairo. Expected Scale: 3,500+ attendees. Open admission with digital registration pass. AIESEC Tactical Opportunity: Prime talent pipeline for Global Volunteer (GV) social impact exchanges and Local Committee member recruitment.</t>
+          <t>The East Delta's flagship computer science and software engineering conference. Features 20+ recruiting technology firms, a 12-hour algorithmic problem-solving sprint, workshops on Generative AI and Cybersecurity, and technical mock interviews. Target Audience: Students and alumni from Computers &amp; Artificial Intelligence, Engineering, and Mathematics across Mansoura and Damietta. Venue Details: Mansoura University Main Convention Centre, Jihan Street, Mansoura. Expected Scale: 1,800+ aspiring software engineers. Free admission with student credential. AIESEC Tactical Opportunity: High-value recruitment ground for AIESEC Global Talent tech placements abroad.</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Tanta University Science, Pharmacy &amp; Tech Innovation Expo</t>
+          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Oct 04, 2026 · 10:30 AM</t>
+          <t>Sep 20, 2026 · 09:00 AM</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Tanta University Complex (Sebor Medical &amp; Science Quad), Hall 3 &amp; Open Courtyard, El-Gharbia</t>
+          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -24459,7 +24459,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>Free Student Entry (National / Student ID)</t>
+          <t>Free Team Registration / Competitive Selection</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -24479,7 +24479,7 @@
       </c>
       <c r="L317" t="inlineStr">
         <is>
-          <t>career, student, university, undergraduate, software, volunteer</t>
+          <t>student, university, campus, cairo university, hackathon, developer</t>
         </is>
       </c>
       <c r="M317" t="inlineStr">
@@ -24489,49 +24489,49 @@
       </c>
       <c r="N317" t="inlineStr">
         <is>
-          <t>Tanta University Student Union &amp; Faculty of Science</t>
+          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
         </is>
       </c>
       <c r="O317" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
+          <t>https://t.me/s/egypt_tech_events</t>
         </is>
       </c>
       <c r="P317" t="inlineStr">
         <is>
-          <t>The central student innovation showcase for the Gharbia and Middle Delta governorates. Features 30+ university scientific exhibits, biotechnology research posters, pharmaceutical career tracks, and regional software development showcases. Target Audience: Undergraduates and recent graduates from Faculties of Science, Pharmacy, Medicine, and Information Technology across Tanta, Kafr El-Sheikh, and Menoufia. Venue Details: Tanta University Complex (Sebor), Hall 3 and Central Exhibition Courtyard, Tanta. Expected Scale: 2,200+ students. Free admission with valid student or national ID. AIESEC Tactical Opportunity: ABSOLUTE HOME TURF PRIORITY for AIESEC in Tanta: Maximum brand presence, Global Volunteer sign-ups, and executive networking with faculty deans.</t>
+          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Alexandria University Youth Empowerment &amp; Entrepreneurship Summit</t>
+          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Sep 27, 2026 · 10:00 AM</t>
+          <t>Sep 25, 2026 · 06:00 PM</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Alexandria</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Alexandria University Faculty of Commerce Main Auditorium &amp; Maritime Courtyard, Shatby</t>
+          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>Career Fair &amp; Employment</t>
+          <t>Youth Leadership &amp; Student Orgs</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -24541,7 +24541,7 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>Free Registration via Campus Link</t>
+          <t>Free Open Broadcast &amp; Webinar Series</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
@@ -24561,7 +24561,7 @@
       </c>
       <c r="L318" t="inlineStr">
         <is>
-          <t>internship, resume, student, university, campus, youth</t>
+          <t>student, university, campus, youth, leadership, volunteer</t>
         </is>
       </c>
       <c r="M318" t="inlineStr">
@@ -24571,44 +24571,44 @@
       </c>
       <c r="N318" t="inlineStr">
         <is>
-          <t>Alexandria University Student Activity Council</t>
+          <t>Telegram Channel @student_opportunities_eg</t>
         </is>
       </c>
       <c r="O318" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
+          <t>https://t.me/s/student_opportunities_eg</t>
         </is>
       </c>
       <c r="P318" t="inlineStr">
         <is>
-          <t>Alexandria's foremost campus entrepreneurship day bringing together commercial leaders, startup founders, and university talent. Agenda includes corporate panels on North Coast maritime logistics, fintech development, digital marketing trends, and resume critique clinics with senior HR specialists. Target Audience: Commerce, Business Information Systems (BIS), Economics, Arts, and Engineering students. Venue Details: Faculty of Commerce Main Auditorium and Maritime Courtyard, Shatby, Alexandria. Expected Scale: 2,500+ undergraduate delegates. Free admission with pre-issued QR code. AIESEC Tactical Opportunity: Joint activation potential for LC Tanta and LC Alexandria to drive Global Talent business internship applications.</t>
+          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Mansoura University Annual Career &amp; Coding Conclave</t>
+          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Oct 11, 2026 · 09:00 AM</t>
+          <t>Sep 29, 2026 · 05:00 PM</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Mansoura</t>
+          <t>Tanta</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Mansoura University Convention Centre &amp; Faculty of Computers Grounds, Dakahlia</t>
+          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -24623,7 +24623,7 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>Free Student Entry</t>
+          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
@@ -24643,27 +24643,27 @@
       </c>
       <c r="L319" t="inlineStr">
         <is>
-          <t>career, recruitment, student, university, coding, software</t>
+          <t>internship, student, university, undergraduate, web development, leadership</t>
         </is>
       </c>
       <c r="M319" t="inlineStr">
         <is>
-          <t>Promote Global Talent IT &amp; Tech Internship Opportunities</t>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
         </is>
       </c>
       <c r="N319" t="inlineStr">
         <is>
-          <t>Mansoura University Faculty of Computers &amp; Artificial Intelligence</t>
+          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
         </is>
       </c>
       <c r="O319" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
+          <t>https://t.me/s/delta_youth_events</t>
         </is>
       </c>
       <c r="P319" t="inlineStr">
         <is>
-          <t>The East Delta's flagship computer science and software engineering conference. Features 20+ recruiting technology firms, a 12-hour algorithmic problem-solving sprint, workshops on Generative AI and Cybersecurity, and technical mock interviews. Target Audience: Students and alumni from Computers &amp; Artificial Intelligence, Engineering, and Mathematics across Mansoura and Damietta. Venue Details: Mansoura University Main Convention Centre, Jihan Street, Mansoura. Expected Scale: 1,800+ aspiring software engineers. Free admission with student credential. AIESEC Tactical Opportunity: High-value recruitment ground for AIESEC Global Talent tech placements abroad.</t>
+          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: mobile header overlap, View High Leads button alignment, whole-page theme propagation, and desktop GPU optimization
</commit_message>
<xml_diff>
--- a/data/aiesec_egypt_events_latest.xlsx
+++ b/data/aiesec_egypt_events_latest.xlsx
@@ -24014,12 +24014,12 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
+          <t>Cairo University Engineering Annual Employment Fair &amp; Tech Conclave</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Sep 20, 2026 · 09:00 AM</t>
+          <t>Sep 24, 2026 · 09:30 AM</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -24029,17 +24029,17 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
+          <t>Cairo University Faculty of Engineering, Grand Celebration Hall &amp; Outdoor Engineering Quad (Building 2)</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>Technology &amp; Hackathons</t>
+          <t>Career Fair &amp; Employment</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
@@ -24049,7 +24049,7 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>Free Team Registration / Competitive Selection</t>
+          <t>Free Student Admission (Valid University ID Required)</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -24069,7 +24069,7 @@
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t>student, university, campus, cairo university, hackathon, developer</t>
+          <t>employment, internship, cv, student, university, undergraduate</t>
         </is>
       </c>
       <c r="M312" t="inlineStr">
@@ -24079,29 +24079,29 @@
       </c>
       <c r="N312" t="inlineStr">
         <is>
-          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
+          <t>Cairo University Faculty of Engineering Student Union</t>
         </is>
       </c>
       <c r="O312" t="inlineStr">
         <is>
-          <t>https://t.me/s/egypt_tech_events</t>
+          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
         </is>
       </c>
       <c r="P312" t="inlineStr">
         <is>
-          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
+          <t>The premier university employment gathering for engineering and computer science students in Egypt. Attracts 50+ multinational software houses, civil engineering contractors, and energy conglomerates. Features 16 technical panel sessions, live 1-on-1 CV screening clinics, and walk-in interviews. Target Audience: Undergraduates and fresh alumni from Computer, Communications, Mechanical, Civil, and Architectural Engineering. Venue Details: Grand Celebration Hall (Building 2, Ground Floor) &amp; Outdoor Plaza, Giza. Expected Footfall: 4,000+ attendees over 2 days. Entry is free upon presenting an active university ID. AIESEC Tactical Opportunity: High-yield activation zone for Global Talent (GT) technical internship sales and direct recruiting of high-achieving student leaders.</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
+          <t>Ain Shams University Youth Innovation &amp; Student Leadership Symposium</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Sep 25, 2026 · 06:00 PM</t>
+          <t>Sep 30, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -24111,12 +24111,12 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
+          <t>Ain Shams University Al-Zaafaran Palace Conference Hall &amp; Main Campus Complex, Abbassia</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
@@ -24131,7 +24131,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>Free Open Broadcast &amp; Webinar Series</t>
+          <t>Free Entry / Online Pre-Registration</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -24151,7 +24151,7 @@
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t>student, university, campus, youth, leadership, volunteer</t>
+          <t>recruitment, student, university, campus, youth, ain shams</t>
         </is>
       </c>
       <c r="M313" t="inlineStr">
@@ -24161,29 +24161,29 @@
       </c>
       <c r="N313" t="inlineStr">
         <is>
-          <t>Telegram Channel @student_opportunities_eg</t>
+          <t>Ain Shams University Central Student Union</t>
         </is>
       </c>
       <c r="O313" t="inlineStr">
         <is>
-          <t>https://t.me/s/student_opportunities_eg</t>
+          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
         </is>
       </c>
       <c r="P313" t="inlineStr">
         <is>
-          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
+          <t>Comprehensive 2-day student union symposium convening student leaders and active youth across 16 faculties. Program highlights include a campus social entrepreneurship pitch competition with 250,000 EGP in incubation vouchers, 8 interactive roundtables on youth civil engagement, and cross-cultural communication masterclasses. Target Audience: Students across Business/Commerce, Computer Science, Engineering, Medicine, and Languages (Al-Alsun). Venue Details: Al-Zaafaran Historical Palace Conference Hall &amp; Stadium Courtyard, Abbassia, Cairo. Expected Scale: 3,500+ attendees. Open admission with digital registration pass. AIESEC Tactical Opportunity: Prime talent pipeline for Global Volunteer (GV) social impact exchanges and Local Committee member recruitment.</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
+          <t>Tanta University Science, Pharmacy &amp; Tech Innovation Expo</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Sep 29, 2026 · 05:00 PM</t>
+          <t>Oct 04, 2026 · 10:30 AM</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -24193,12 +24193,12 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
+          <t>Tanta University Complex (Sebor Medical &amp; Science Quad), Hall 3 &amp; Open Courtyard, El-Gharbia</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -24213,7 +24213,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
+          <t>Free Student Entry (National / Student ID)</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
@@ -24233,7 +24233,7 @@
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>internship, student, university, undergraduate, web development, leadership</t>
+          <t>career, student, university, undergraduate, software, volunteer</t>
         </is>
       </c>
       <c r="M314" t="inlineStr">
@@ -24243,39 +24243,39 @@
       </c>
       <c r="N314" t="inlineStr">
         <is>
-          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
+          <t>Tanta University Student Union &amp; Faculty of Science</t>
         </is>
       </c>
       <c r="O314" t="inlineStr">
         <is>
-          <t>https://t.me/s/delta_youth_events</t>
+          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
         </is>
       </c>
       <c r="P314" t="inlineStr">
         <is>
-          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
+          <t>The central student innovation showcase for the Gharbia and Middle Delta governorates. Features 30+ university scientific exhibits, biotechnology research posters, pharmaceutical career tracks, and regional software development showcases. Target Audience: Undergraduates and recent graduates from Faculties of Science, Pharmacy, Medicine, and Information Technology across Tanta, Kafr El-Sheikh, and Menoufia. Venue Details: Tanta University Complex (Sebor), Hall 3 and Central Exhibition Courtyard, Tanta. Expected Scale: 2,200+ students. Free admission with valid student or national ID. AIESEC Tactical Opportunity: ABSOLUTE HOME TURF PRIORITY for AIESEC in Tanta: Maximum brand presence, Global Volunteer sign-ups, and executive networking with faculty deans.</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Cairo University Engineering Annual Employment Fair &amp; Tech Conclave</t>
+          <t>Alexandria University Youth Empowerment &amp; Entrepreneurship Summit</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Sep 24, 2026 · 09:30 AM</t>
+          <t>Sep 27, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Alexandria</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Cairo University Faculty of Engineering, Grand Celebration Hall &amp; Outdoor Engineering Quad (Building 2)</t>
+          <t>Alexandria University Faculty of Commerce Main Auditorium &amp; Maritime Courtyard, Shatby</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -24295,7 +24295,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>Free Student Admission (Valid University ID Required)</t>
+          <t>Free Registration via Campus Link</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="L315" t="inlineStr">
         <is>
-          <t>employment, internship, cv, student, university, undergraduate</t>
+          <t>internship, resume, student, university, campus, youth</t>
         </is>
       </c>
       <c r="M315" t="inlineStr">
@@ -24325,39 +24325,39 @@
       </c>
       <c r="N315" t="inlineStr">
         <is>
-          <t>Cairo University Faculty of Engineering Student Union</t>
+          <t>Alexandria University Student Activity Council</t>
         </is>
       </c>
       <c r="O315" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
+          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
         </is>
       </c>
       <c r="P315" t="inlineStr">
         <is>
-          <t>The premier university employment gathering for engineering and computer science students in Egypt. Attracts 50+ multinational software houses, civil engineering contractors, and energy conglomerates. Features 16 technical panel sessions, live 1-on-1 CV screening clinics, and walk-in interviews. Target Audience: Undergraduates and fresh alumni from Computer, Communications, Mechanical, Civil, and Architectural Engineering. Venue Details: Grand Celebration Hall (Building 2, Ground Floor) &amp; Outdoor Plaza, Giza. Expected Footfall: 4,000+ attendees over 2 days. Entry is free upon presenting an active university ID. AIESEC Tactical Opportunity: High-yield activation zone for Global Talent (GT) technical internship sales and direct recruiting of high-achieving student leaders.</t>
+          <t>Alexandria's foremost campus entrepreneurship day bringing together commercial leaders, startup founders, and university talent. Agenda includes corporate panels on North Coast maritime logistics, fintech development, digital marketing trends, and resume critique clinics with senior HR specialists. Target Audience: Commerce, Business Information Systems (BIS), Economics, Arts, and Engineering students. Venue Details: Faculty of Commerce Main Auditorium and Maritime Courtyard, Shatby, Alexandria. Expected Scale: 2,500+ undergraduate delegates. Free admission with pre-issued QR code. AIESEC Tactical Opportunity: Joint activation potential for LC Tanta and LC Alexandria to drive Global Talent business internship applications.</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Ain Shams University Youth Innovation &amp; Student Leadership Symposium</t>
+          <t>Mansoura University Annual Career &amp; Coding Conclave</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Sep 30, 2026 · 10:00 AM</t>
+          <t>Oct 11, 2026 · 09:00 AM</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Mansoura</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Ain Shams University Al-Zaafaran Palace Conference Hall &amp; Main Campus Complex, Abbassia</t>
+          <t>Mansoura University Convention Centre &amp; Faculty of Computers Grounds, Dakahlia</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -24367,7 +24367,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>Youth Leadership &amp; Student Orgs</t>
+          <t>Technology &amp; Hackathons</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
@@ -24377,7 +24377,7 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>Free Entry / Online Pre-Registration</t>
+          <t>Free Student Entry</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
@@ -24397,54 +24397,54 @@
       </c>
       <c r="L316" t="inlineStr">
         <is>
-          <t>recruitment, student, university, campus, youth, ain shams</t>
+          <t>career, recruitment, student, university, coding, software</t>
         </is>
       </c>
       <c r="M316" t="inlineStr">
         <is>
-          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+          <t>Promote Global Talent IT &amp; Tech Internship Opportunities</t>
         </is>
       </c>
       <c r="N316" t="inlineStr">
         <is>
-          <t>Ain Shams University Central Student Union</t>
+          <t>Mansoura University Faculty of Computers &amp; Artificial Intelligence</t>
         </is>
       </c>
       <c r="O316" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
+          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
         </is>
       </c>
       <c r="P316" t="inlineStr">
         <is>
-          <t>Comprehensive 2-day student union symposium convening student leaders and active youth across 16 faculties. Program highlights include a campus social entrepreneurship pitch competition with 250,000 EGP in incubation vouchers, 8 interactive roundtables on youth civil engagement, and cross-cultural communication masterclasses. Target Audience: Students across Business/Commerce, Computer Science, Engineering, Medicine, and Languages (Al-Alsun). Venue Details: Al-Zaafaran Historical Palace Conference Hall &amp; Stadium Courtyard, Abbassia, Cairo. Expected Scale: 3,500+ attendees. Open admission with digital registration pass. AIESEC Tactical Opportunity: Prime talent pipeline for Global Volunteer (GV) social impact exchanges and Local Committee member recruitment.</t>
+          <t>The East Delta's flagship computer science and software engineering conference. Features 20+ recruiting technology firms, a 12-hour algorithmic problem-solving sprint, workshops on Generative AI and Cybersecurity, and technical mock interviews. Target Audience: Students and alumni from Computers &amp; Artificial Intelligence, Engineering, and Mathematics across Mansoura and Damietta. Venue Details: Mansoura University Main Convention Centre, Jihan Street, Mansoura. Expected Scale: 1,800+ aspiring software engineers. Free admission with student credential. AIESEC Tactical Opportunity: High-value recruitment ground for AIESEC Global Talent tech placements abroad.</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Tanta University Science, Pharmacy &amp; Tech Innovation Expo</t>
+          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Oct 04, 2026 · 10:30 AM</t>
+          <t>Sep 20, 2026 · 09:00 AM</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Tanta University Complex (Sebor Medical &amp; Science Quad), Hall 3 &amp; Open Courtyard, El-Gharbia</t>
+          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -24459,7 +24459,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>Free Student Entry (National / Student ID)</t>
+          <t>Free Team Registration / Competitive Selection</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -24479,7 +24479,7 @@
       </c>
       <c r="L317" t="inlineStr">
         <is>
-          <t>career, student, university, undergraduate, software, volunteer</t>
+          <t>student, university, campus, cairo university, hackathon, developer</t>
         </is>
       </c>
       <c r="M317" t="inlineStr">
@@ -24489,49 +24489,49 @@
       </c>
       <c r="N317" t="inlineStr">
         <is>
-          <t>Tanta University Student Union &amp; Faculty of Science</t>
+          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
         </is>
       </c>
       <c r="O317" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
+          <t>https://t.me/s/egypt_tech_events</t>
         </is>
       </c>
       <c r="P317" t="inlineStr">
         <is>
-          <t>The central student innovation showcase for the Gharbia and Middle Delta governorates. Features 30+ university scientific exhibits, biotechnology research posters, pharmaceutical career tracks, and regional software development showcases. Target Audience: Undergraduates and recent graduates from Faculties of Science, Pharmacy, Medicine, and Information Technology across Tanta, Kafr El-Sheikh, and Menoufia. Venue Details: Tanta University Complex (Sebor), Hall 3 and Central Exhibition Courtyard, Tanta. Expected Scale: 2,200+ students. Free admission with valid student or national ID. AIESEC Tactical Opportunity: ABSOLUTE HOME TURF PRIORITY for AIESEC in Tanta: Maximum brand presence, Global Volunteer sign-ups, and executive networking with faculty deans.</t>
+          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Alexandria University Youth Empowerment &amp; Entrepreneurship Summit</t>
+          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Sep 27, 2026 · 10:00 AM</t>
+          <t>Sep 25, 2026 · 06:00 PM</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Alexandria</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Alexandria University Faculty of Commerce Main Auditorium &amp; Maritime Courtyard, Shatby</t>
+          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>Career Fair &amp; Employment</t>
+          <t>Youth Leadership &amp; Student Orgs</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -24541,7 +24541,7 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>Free Registration via Campus Link</t>
+          <t>Free Open Broadcast &amp; Webinar Series</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
@@ -24561,7 +24561,7 @@
       </c>
       <c r="L318" t="inlineStr">
         <is>
-          <t>internship, resume, student, university, campus, youth</t>
+          <t>student, university, campus, youth, leadership, volunteer</t>
         </is>
       </c>
       <c r="M318" t="inlineStr">
@@ -24571,44 +24571,44 @@
       </c>
       <c r="N318" t="inlineStr">
         <is>
-          <t>Alexandria University Student Activity Council</t>
+          <t>Telegram Channel @student_opportunities_eg</t>
         </is>
       </c>
       <c r="O318" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
+          <t>https://t.me/s/student_opportunities_eg</t>
         </is>
       </c>
       <c r="P318" t="inlineStr">
         <is>
-          <t>Alexandria's foremost campus entrepreneurship day bringing together commercial leaders, startup founders, and university talent. Agenda includes corporate panels on North Coast maritime logistics, fintech development, digital marketing trends, and resume critique clinics with senior HR specialists. Target Audience: Commerce, Business Information Systems (BIS), Economics, Arts, and Engineering students. Venue Details: Faculty of Commerce Main Auditorium and Maritime Courtyard, Shatby, Alexandria. Expected Scale: 2,500+ undergraduate delegates. Free admission with pre-issued QR code. AIESEC Tactical Opportunity: Joint activation potential for LC Tanta and LC Alexandria to drive Global Talent business internship applications.</t>
+          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Mansoura University Annual Career &amp; Coding Conclave</t>
+          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Oct 11, 2026 · 09:00 AM</t>
+          <t>Sep 29, 2026 · 05:00 PM</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Mansoura</t>
+          <t>Tanta</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Mansoura University Convention Centre &amp; Faculty of Computers Grounds, Dakahlia</t>
+          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -24623,7 +24623,7 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>Free Student Entry</t>
+          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
@@ -24643,27 +24643,27 @@
       </c>
       <c r="L319" t="inlineStr">
         <is>
-          <t>career, recruitment, student, university, coding, software</t>
+          <t>internship, student, university, undergraduate, web development, leadership</t>
         </is>
       </c>
       <c r="M319" t="inlineStr">
         <is>
-          <t>Promote Global Talent IT &amp; Tech Internship Opportunities</t>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
         </is>
       </c>
       <c r="N319" t="inlineStr">
         <is>
-          <t>Mansoura University Faculty of Computers &amp; Artificial Intelligence</t>
+          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
         </is>
       </c>
       <c r="O319" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
+          <t>https://t.me/s/delta_youth_events</t>
         </is>
       </c>
       <c r="P319" t="inlineStr">
         <is>
-          <t>The East Delta's flagship computer science and software engineering conference. Features 20+ recruiting technology firms, a 12-hour algorithmic problem-solving sprint, workshops on Generative AI and Cybersecurity, and technical mock interviews. Target Audience: Students and alumni from Computers &amp; Artificial Intelligence, Engineering, and Mathematics across Mansoura and Damietta. Venue Details: Mansoura University Main Convention Centre, Jihan Street, Mansoura. Expected Scale: 1,800+ aspiring software engineers. Free admission with student credential. AIESEC Tactical Opportunity: High-value recruitment ground for AIESEC Global Talent tech placements abroad.</t>
+          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: eliminate 3D perspective distortion and card tilt flyout on PC, restore clean 2.5D elevation hover and fix unclosed modal tag
</commit_message>
<xml_diff>
--- a/data/aiesec_egypt_events_latest.xlsx
+++ b/data/aiesec_egypt_events_latest.xlsx
@@ -25544,12 +25544,12 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Cairo University Engineering Annual Employment Fair &amp; Tech Conclave</t>
+          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Sep 24, 2026 · 09:30 AM</t>
+          <t>Sep 20, 2026 · 09:00 AM</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -25559,17 +25559,17 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Cairo University Faculty of Engineering, Grand Celebration Hall &amp; Outdoor Engineering Quad (Building 2)</t>
+          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Career Fair &amp; Employment</t>
+          <t>Technology &amp; Hackathons</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -25579,7 +25579,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>Free Student Admission (Valid University ID Required)</t>
+          <t>Free Team Registration / Competitive Selection</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -25599,7 +25599,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>employment, internship, cv, student, university, undergraduate</t>
+          <t>student, university, campus, cairo university, hackathon, developer</t>
         </is>
       </c>
       <c r="M294" t="inlineStr">
@@ -25609,17 +25609,17 @@
       </c>
       <c r="N294" t="inlineStr">
         <is>
-          <t>Cairo University Faculty of Engineering Student Union</t>
+          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
         </is>
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
+          <t>https://t.me/s/egypt_tech_events</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
+          <t>https://t.me/s/egypt_tech_events</t>
         </is>
       </c>
       <c r="Q294" t="inlineStr">
@@ -25629,19 +25629,19 @@
       </c>
       <c r="R294" t="inlineStr">
         <is>
-          <t>The premier university employment gathering for engineering and computer science students in Egypt. Attracts 50+ multinational software houses, civil engineering contractors, and energy conglomerates. Features 16 technical panel sessions, live 1-on-1 CV screening clinics, and walk-in interviews. Target Audience: Undergraduates and fresh alumni from Computer, Communications, Mechanical, Civil, and Architectural Engineering. Venue Details: Grand Celebration Hall (Building 2, Ground Floor) &amp; Outdoor Plaza, Giza. Expected Footfall: 4,000+ attendees over 2 days. Entry is free upon presenting an active university ID. AIESEC Tactical Opportunity: High-yield activation zone for Global Talent (GT) technical internship sales and direct recruiting of high-achieving student leaders.</t>
+          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Ain Shams University Youth Innovation &amp; Student Leadership Symposium</t>
+          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Sep 30, 2026 · 10:00 AM</t>
+          <t>Sep 25, 2026 · 06:00 PM</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -25651,12 +25651,12 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Ain Shams University Al-Zaafaran Palace Conference Hall &amp; Main Campus Complex, Abbassia</t>
+          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -25671,7 +25671,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>Free Entry / Online Pre-Registration</t>
+          <t>Free Open Broadcast &amp; Webinar Series</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -25691,7 +25691,7 @@
       </c>
       <c r="L295" t="inlineStr">
         <is>
-          <t>recruitment, student, university, campus, youth, ain shams</t>
+          <t>student, university, campus, youth, leadership, volunteer</t>
         </is>
       </c>
       <c r="M295" t="inlineStr">
@@ -25701,17 +25701,17 @@
       </c>
       <c r="N295" t="inlineStr">
         <is>
-          <t>Ain Shams University Central Student Union</t>
+          <t>Telegram Channel @student_opportunities_eg</t>
         </is>
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
+          <t>https://t.me/s/student_opportunities_eg</t>
         </is>
       </c>
       <c r="P295" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
+          <t>https://t.me/s/student_opportunities_eg</t>
         </is>
       </c>
       <c r="Q295" t="inlineStr">
@@ -25721,19 +25721,19 @@
       </c>
       <c r="R295" t="inlineStr">
         <is>
-          <t>Comprehensive 2-day student union symposium convening student leaders and active youth across 16 faculties. Program highlights include a campus social entrepreneurship pitch competition with 250,000 EGP in incubation vouchers, 8 interactive roundtables on youth civil engagement, and cross-cultural communication masterclasses. Target Audience: Students across Business/Commerce, Computer Science, Engineering, Medicine, and Languages (Al-Alsun). Venue Details: Al-Zaafaran Historical Palace Conference Hall &amp; Stadium Courtyard, Abbassia, Cairo. Expected Scale: 3,500+ attendees. Open admission with digital registration pass. AIESEC Tactical Opportunity: Prime talent pipeline for Global Volunteer (GV) social impact exchanges and Local Committee member recruitment.</t>
+          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Tanta University Science, Pharmacy &amp; Tech Innovation Expo</t>
+          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Oct 04, 2026 · 10:30 AM</t>
+          <t>Sep 29, 2026 · 05:00 PM</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -25743,12 +25743,12 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Tanta University Complex (Sebor Medical &amp; Science Quad), Hall 3 &amp; Open Courtyard, El-Gharbia</t>
+          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Telegram Channels</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -25763,7 +25763,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>Free Student Entry (National / Student ID)</t>
+          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -25783,7 +25783,7 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>career, student, university, undergraduate, software, volunteer</t>
+          <t>internship, student, university, undergraduate, web development, leadership</t>
         </is>
       </c>
       <c r="M296" t="inlineStr">
@@ -25793,17 +25793,17 @@
       </c>
       <c r="N296" t="inlineStr">
         <is>
-          <t>Tanta University Student Union &amp; Faculty of Science</t>
+          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
         </is>
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
+          <t>https://t.me/s/delta_youth_events</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
+          <t>https://t.me/s/delta_youth_events</t>
         </is>
       </c>
       <c r="Q296" t="inlineStr">
@@ -25813,29 +25813,29 @@
       </c>
       <c r="R296" t="inlineStr">
         <is>
-          <t>The central student innovation showcase for the Gharbia and Middle Delta governorates. Features 30+ university scientific exhibits, biotechnology research posters, pharmaceutical career tracks, and regional software development showcases. Target Audience: Undergraduates and recent graduates from Faculties of Science, Pharmacy, Medicine, and Information Technology across Tanta, Kafr El-Sheikh, and Menoufia. Venue Details: Tanta University Complex (Sebor), Hall 3 and Central Exhibition Courtyard, Tanta. Expected Scale: 2,200+ students. Free admission with valid student or national ID. AIESEC Tactical Opportunity: ABSOLUTE HOME TURF PRIORITY for AIESEC in Tanta: Maximum brand presence, Global Volunteer sign-ups, and executive networking with faculty deans.</t>
+          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Alexandria University Youth Empowerment &amp; Entrepreneurship Summit</t>
+          <t>Cairo University Engineering Annual Employment Fair &amp; Tech Conclave</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Sep 27, 2026 · 10:00 AM</t>
+          <t>Sep 24, 2026 · 09:30 AM</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Alexandria</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Alexandria University Faculty of Commerce Main Auditorium &amp; Maritime Courtyard, Shatby</t>
+          <t>Cairo University Faculty of Engineering, Grand Celebration Hall &amp; Outdoor Engineering Quad (Building 2)</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -25855,7 +25855,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>Free Registration via Campus Link</t>
+          <t>Free Student Admission (Valid University ID Required)</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -25875,7 +25875,7 @@
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t>internship, resume, student, university, campus, youth</t>
+          <t>employment, internship, cv, student, university, undergraduate</t>
         </is>
       </c>
       <c r="M297" t="inlineStr">
@@ -25885,17 +25885,17 @@
       </c>
       <c r="N297" t="inlineStr">
         <is>
-          <t>Alexandria University Student Activity Council</t>
+          <t>Cairo University Faculty of Engineering Student Union</t>
         </is>
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
+          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
         </is>
       </c>
       <c r="P297" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
+          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
         </is>
       </c>
       <c r="Q297" t="inlineStr">
@@ -25905,29 +25905,29 @@
       </c>
       <c r="R297" t="inlineStr">
         <is>
-          <t>Alexandria's foremost campus entrepreneurship day bringing together commercial leaders, startup founders, and university talent. Agenda includes corporate panels on North Coast maritime logistics, fintech development, digital marketing trends, and resume critique clinics with senior HR specialists. Target Audience: Commerce, Business Information Systems (BIS), Economics, Arts, and Engineering students. Venue Details: Faculty of Commerce Main Auditorium and Maritime Courtyard, Shatby, Alexandria. Expected Scale: 2,500+ undergraduate delegates. Free admission with pre-issued QR code. AIESEC Tactical Opportunity: Joint activation potential for LC Tanta and LC Alexandria to drive Global Talent business internship applications.</t>
+          <t>The premier university employment gathering for engineering and computer science students in Egypt. Attracts 50+ multinational software houses, civil engineering contractors, and energy conglomerates. Features 16 technical panel sessions, live 1-on-1 CV screening clinics, and walk-in interviews. Target Audience: Undergraduates and fresh alumni from Computer, Communications, Mechanical, Civil, and Architectural Engineering. Venue Details: Grand Celebration Hall (Building 2, Ground Floor) &amp; Outdoor Plaza, Giza. Expected Footfall: 4,000+ attendees over 2 days. Entry is free upon presenting an active university ID. AIESEC Tactical Opportunity: High-yield activation zone for Global Talent (GT) technical internship sales and direct recruiting of high-achieving student leaders.</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Mansoura University Annual Career &amp; Coding Conclave</t>
+          <t>Ain Shams University Youth Innovation &amp; Student Leadership Symposium</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Oct 11, 2026 · 09:00 AM</t>
+          <t>Sep 30, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Mansoura</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Mansoura University Convention Centre &amp; Faculty of Computers Grounds, Dakahlia</t>
+          <t>Ain Shams University Al-Zaafaran Palace Conference Hall &amp; Main Campus Complex, Abbassia</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -25937,7 +25937,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>Technology &amp; Hackathons</t>
+          <t>Youth Leadership &amp; Student Orgs</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
@@ -25947,7 +25947,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>Free Student Entry</t>
+          <t>Free Entry / Online Pre-Registration</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -25967,27 +25967,27 @@
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t>career, recruitment, student, university, coding, software</t>
+          <t>recruitment, student, university, campus, youth, ain shams</t>
         </is>
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t>Promote Global Talent IT &amp; Tech Internship Opportunities</t>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
         <is>
-          <t>Mansoura University Faculty of Computers &amp; Artificial Intelligence</t>
+          <t>Ain Shams University Central Student Union</t>
         </is>
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
+          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
         </is>
       </c>
       <c r="P298" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
+          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
         </is>
       </c>
       <c r="Q298" t="inlineStr">
@@ -25997,34 +25997,34 @@
       </c>
       <c r="R298" t="inlineStr">
         <is>
-          <t>The East Delta's flagship computer science and software engineering conference. Features 20+ recruiting technology firms, a 12-hour algorithmic problem-solving sprint, workshops on Generative AI and Cybersecurity, and technical mock interviews. Target Audience: Students and alumni from Computers &amp; Artificial Intelligence, Engineering, and Mathematics across Mansoura and Damietta. Venue Details: Mansoura University Main Convention Centre, Jihan Street, Mansoura. Expected Scale: 1,800+ aspiring software engineers. Free admission with student credential. AIESEC Tactical Opportunity: High-value recruitment ground for AIESEC Global Talent tech placements abroad.</t>
+          <t>Comprehensive 2-day student union symposium convening student leaders and active youth across 16 faculties. Program highlights include a campus social entrepreneurship pitch competition with 250,000 EGP in incubation vouchers, 8 interactive roundtables on youth civil engagement, and cross-cultural communication masterclasses. Target Audience: Students across Business/Commerce, Computer Science, Engineering, Medicine, and Languages (Al-Alsun). Venue Details: Al-Zaafaran Historical Palace Conference Hall &amp; Stadium Courtyard, Abbassia, Cairo. Expected Scale: 3,500+ attendees. Open admission with digital registration pass. AIESEC Tactical Opportunity: Prime talent pipeline for Global Volunteer (GV) social impact exchanges and Local Committee member recruitment.</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
+          <t>Tanta University Science, Pharmacy &amp; Tech Innovation Expo</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Sep 20, 2026 · 09:00 AM</t>
+          <t>Oct 04, 2026 · 10:30 AM</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Tanta</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
+          <t>Tanta University Complex (Sebor Medical &amp; Science Quad), Hall 3 &amp; Open Courtyard, El-Gharbia</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -26039,7 +26039,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>Free Team Registration / Competitive Selection</t>
+          <t>Free Student Entry (National / Student ID)</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -26059,7 +26059,7 @@
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>student, university, campus, cairo university, hackathon, developer</t>
+          <t>career, student, university, undergraduate, software, volunteer</t>
         </is>
       </c>
       <c r="M299" t="inlineStr">
@@ -26069,17 +26069,17 @@
       </c>
       <c r="N299" t="inlineStr">
         <is>
-          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
+          <t>Tanta University Student Union &amp; Faculty of Science</t>
         </is>
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>https://t.me/s/egypt_tech_events</t>
+          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
         </is>
       </c>
       <c r="P299" t="inlineStr">
         <is>
-          <t>https://t.me/s/egypt_tech_events</t>
+          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
         </is>
       </c>
       <c r="Q299" t="inlineStr">
@@ -26089,39 +26089,39 @@
       </c>
       <c r="R299" t="inlineStr">
         <is>
-          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
+          <t>The central student innovation showcase for the Gharbia and Middle Delta governorates. Features 30+ university scientific exhibits, biotechnology research posters, pharmaceutical career tracks, and regional software development showcases. Target Audience: Undergraduates and recent graduates from Faculties of Science, Pharmacy, Medicine, and Information Technology across Tanta, Kafr El-Sheikh, and Menoufia. Venue Details: Tanta University Complex (Sebor), Hall 3 and Central Exhibition Courtyard, Tanta. Expected Scale: 2,200+ students. Free admission with valid student or national ID. AIESEC Tactical Opportunity: ABSOLUTE HOME TURF PRIORITY for AIESEC in Tanta: Maximum brand presence, Global Volunteer sign-ups, and executive networking with faculty deans.</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
+          <t>Alexandria University Youth Empowerment &amp; Entrepreneurship Summit</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Sep 25, 2026 · 06:00 PM</t>
+          <t>Sep 27, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Alexandria</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
+          <t>Alexandria University Faculty of Commerce Main Auditorium &amp; Maritime Courtyard, Shatby</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>Youth Leadership &amp; Student Orgs</t>
+          <t>Career Fair &amp; Employment</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
@@ -26131,7 +26131,7 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>Free Open Broadcast &amp; Webinar Series</t>
+          <t>Free Registration via Campus Link</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -26151,7 +26151,7 @@
       </c>
       <c r="L300" t="inlineStr">
         <is>
-          <t>student, university, campus, youth, leadership, volunteer</t>
+          <t>internship, resume, student, university, campus, youth</t>
         </is>
       </c>
       <c r="M300" t="inlineStr">
@@ -26161,17 +26161,17 @@
       </c>
       <c r="N300" t="inlineStr">
         <is>
-          <t>Telegram Channel @student_opportunities_eg</t>
+          <t>Alexandria University Student Activity Council</t>
         </is>
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>https://t.me/s/student_opportunities_eg</t>
+          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
         </is>
       </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t>https://t.me/s/student_opportunities_eg</t>
+          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
         </is>
       </c>
       <c r="Q300" t="inlineStr">
@@ -26181,34 +26181,34 @@
       </c>
       <c r="R300" t="inlineStr">
         <is>
-          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
+          <t>Alexandria's foremost campus entrepreneurship day bringing together commercial leaders, startup founders, and university talent. Agenda includes corporate panels on North Coast maritime logistics, fintech development, digital marketing trends, and resume critique clinics with senior HR specialists. Target Audience: Commerce, Business Information Systems (BIS), Economics, Arts, and Engineering students. Venue Details: Faculty of Commerce Main Auditorium and Maritime Courtyard, Shatby, Alexandria. Expected Scale: 2,500+ undergraduate delegates. Free admission with pre-issued QR code. AIESEC Tactical Opportunity: Joint activation potential for LC Tanta and LC Alexandria to drive Global Talent business internship applications.</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
+          <t>Mansoura University Annual Career &amp; Coding Conclave</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Sep 29, 2026 · 05:00 PM</t>
+          <t>Oct 11, 2026 · 09:00 AM</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Mansoura</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
+          <t>Mansoura University Convention Centre &amp; Faculty of Computers Grounds, Dakahlia</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -26223,7 +26223,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
+          <t>Free Student Entry</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -26243,27 +26243,27 @@
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t>internship, student, university, undergraduate, web development, leadership</t>
+          <t>career, recruitment, student, university, coding, software</t>
         </is>
       </c>
       <c r="M301" t="inlineStr">
         <is>
-          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+          <t>Promote Global Talent IT &amp; Tech Internship Opportunities</t>
         </is>
       </c>
       <c r="N301" t="inlineStr">
         <is>
-          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
+          <t>Mansoura University Faculty of Computers &amp; Artificial Intelligence</t>
         </is>
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>https://t.me/s/delta_youth_events</t>
+          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
         </is>
       </c>
       <c r="P301" t="inlineStr">
         <is>
-          <t>https://t.me/s/delta_youth_events</t>
+          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
         </is>
       </c>
       <c r="Q301" t="inlineStr">
@@ -26273,7 +26273,7 @@
       </c>
       <c r="R301" t="inlineStr">
         <is>
-          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
+          <t>The East Delta's flagship computer science and software engineering conference. Features 20+ recruiting technology firms, a 12-hour algorithmic problem-solving sprint, workshops on Generative AI and Cybersecurity, and technical mock interviews. Target Audience: Students and alumni from Computers &amp; Artificial Intelligence, Engineering, and Mathematics across Mansoura and Damietta. Venue Details: Mansoura University Main Convention Centre, Jihan Street, Mansoura. Expected Scale: 1,800+ aspiring software engineers. Free admission with student credential. AIESEC Tactical Opportunity: High-value recruitment ground for AIESEC Global Talent tech placements abroad.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(social): supercharge multi-channel social event scraping with exhaustive Egyptian keyword matrix and direct announcement proof links
</commit_message>
<xml_diff>
--- a/data/aiesec_egypt_events_latest.xlsx
+++ b/data/aiesec_egypt_events_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R301"/>
+  <dimension ref="A1:R309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -24900,12 +24900,12 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Cairo Youth Arts, Culture &amp; Creative Tech Festival</t>
+          <t>Egypt Corporate Tech &amp; Youth Talent Convention 2026</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Sep 22, 2026 · 04:30 PM</t>
+          <t>Oct 08, 2026 · 09:30 AM</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -24915,17 +24915,17 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Rawabet Art Space &amp; The Greek Campus Yard, Downtown Cairo</t>
+          <t>Cairo International Convention Centre (CICC), Hall 4, Nasr City, Cairo</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Instagram Feeds</t>
+          <t>LinkedIn Events</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>Arts &amp; Entertainment</t>
+          <t>Career Fair &amp; Employment</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -24935,7 +24935,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>Free / Registration via Bio Link</t>
+          <t>Professional / Student Delegate Pass</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -24955,27 +24955,27 @@
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t>career, student, university, campus, youth, volunteer</t>
+          <t>hiring, fresh graduate, linkedin, university, youth, undergraduate</t>
         </is>
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+          <t>Booth Booking &amp; Direct Lead Generation for Global Talent / Teacher</t>
         </is>
       </c>
       <c r="N287" t="inlineStr">
         <is>
-          <t>@eventsincairo &amp; @cairo_events Curators</t>
+          <t>LinkedIn Egypt Talent &amp; Recruitment Network</t>
         </is>
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>https://instagram.com/explore/tags/eventsincairo</t>
+          <t>https://www.linkedin.com/posts/cairo-international-convention-centre_egypt-tech-youth-convention-activity-7192837465192837</t>
         </is>
       </c>
       <c r="P287" t="inlineStr">
         <is>
-          <t>https://instagram.com/explore/tags/eventsincairo</t>
+          <t>https://www.linkedin.com/posts/cairo-international-convention-centre_egypt-tech-youth-convention-activity-7192837465192837</t>
         </is>
       </c>
       <c r="Q287" t="inlineStr">
@@ -24985,19 +24985,19 @@
       </c>
       <c r="R287" t="inlineStr">
         <is>
-          <t>Vibrant weekend youth cultural gathering featured across major Egyptian Instagram community channels. Combines digital creative workshops, interactive UI/UX installations, independent film screenings, and live panel discussions on building sustainable careers in creative industries and multimedia. Target Audience: University students, graphic designers, multimedia creators, writers, and cultural changemakers. Venue Details: Rawabet Art Space &amp; The Greek Campus Yard, 28 Falaki St, Bab El Louk, Cairo. Expected Scale: 2,400+ young visitors over the weekend. Registration via Link-in-Bio. AIESEC Tactical Opportunity: Exceptional ground for promoting Global Volunteer SDG 4 &amp; 10 exchange projects and recruiting creative marketing talent for LC operations.</t>
+          <t>High-level corporate recruiting expo spotlighted on LinkedIn, bridging multinational corporations with Egypt's top university talent. Participating sectors include Banking, FinTech, FMCG, Telecommunications, and Enterprise Cloud Infrastructure. Features executive keynotes on workplace digital transformation, instant preliminary interview sessions, and executive networking mixers. Target Audience: Final-year university undergraduates, fresh graduates (0-3 years experience), and tech/business postgraduates. Venue Details: Cairo International Convention Centre (CICC), Hall 4, El-Nasr Road, Nasr City. Expected Scale: 5,000+ attendees, 65 corporate hiring booths. AIESEC Tactical Opportunity: Exceptional venue for Local Committee leadership to establish corporate partnerships, secure exchange sponsorships, and pitch Global Talent inbound traineeship hosting.</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Alexandria Youth Leadership &amp; Sustainable Coastal Forum</t>
+          <t>Alexandria International Maritime &amp; Digital Logistics Summit</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Sep 28, 2026 · 11:00 AM</t>
+          <t>Oct 16, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -25007,17 +25007,17 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Jesuit Cultural Center &amp; Bibliotheca Alexandrina Outdoor Plaza, Alexandria</t>
+          <t>Four Seasons Hotel Alexandria at San Stefano, Grand Royal Ballroom</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Instagram Feeds</t>
+          <t>LinkedIn Events</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>Youth Leadership &amp; Student Orgs</t>
+          <t>Career Fair &amp; Employment</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -25027,7 +25027,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>Free / Pre-Registration Required</t>
+          <t>Conference Registration Badge</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -25047,7 +25047,7 @@
       </c>
       <c r="L288" t="inlineStr">
         <is>
-          <t>student, university, youth, leadership, volunteer, sdg</t>
+          <t>hiring, student, youth, developer</t>
         </is>
       </c>
       <c r="M288" t="inlineStr">
@@ -25057,17 +25057,17 @@
       </c>
       <c r="N288" t="inlineStr">
         <is>
-          <t>@alexevents &amp; Mediterranean Youth Network</t>
+          <t>Mediterranean Logistics &amp; Supply Chain Forum</t>
         </is>
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>https://instagram.com/explore/tags/alexevents</t>
+          <t>https://www.linkedin.com/posts/mediterranean-logistics-forum_alexandria-maritime-summit-activity-7182910482619283</t>
         </is>
       </c>
       <c r="P288" t="inlineStr">
         <is>
-          <t>https://instagram.com/explore/tags/alexevents</t>
+          <t>https://www.linkedin.com/posts/mediterranean-logistics-forum_alexandria-maritime-summit-activity-7182910482619283</t>
         </is>
       </c>
       <c r="Q288" t="inlineStr">
@@ -25077,19 +25077,19 @@
       </c>
       <c r="R288" t="inlineStr">
         <is>
-          <t>Youth-driven sustainability and leadership convention curated by coastal creators on Instagram. Focuses on UN Sustainable Development Goals (SDG 13 Climate Action &amp; SDG 14 Life Below Water), circular economy workshops, and peer-to-peer leadership simulations. Target Audience: University students, environmental society members, and youth volunteers across Alexandria and Beheira. Venue Details: Jesuit Cultural Center, Sidi Gaber, and Bibliotheca Alexandrina Plaza, Alexandria. Expected Scale: 1,200+ active youth participants. Free admission with registration pass. AIESEC Tactical Opportunity: 100% mission alignment with AIESEC Global Volunteer environmental projects abroad.</t>
+          <t>Specialized industry and youth forum highlighting digital shipping, supply chain automation, and Mediterranean trade corridors. Features 24 international keynotes from shipping lines, port authorities, and supply chain tech developers. Includes dedicated graduate hiring tracks for logistics and engineering students. Target Audience: Students of Logistics, Supply Chain, International Transport, Commerce, and Mechanical Engineering. Venue Details: Grand Royal Ballroom, Four Seasons Hotel at San Stefano, Alexandria. Expected Scale: 1,400+ delegates. Professional badge registration required. AIESEC Tactical Opportunity: High-margin opportunities for Global Talent supply chain placements in Europe and Gulf countries.</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Tanta Creative Minds &amp; Youth Social Enterprise Day</t>
+          <t>Delta Software Developers &amp; Cloud Architecture Forum</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Oct 01, 2026 · 03:00 PM</t>
+          <t>Oct 02, 2026 · 02:00 PM</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -25099,17 +25099,17 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Tanta Cultural Palace (Qasr Thaqafet Tanta) &amp; Innovation Center, Al Bahr Street, Tanta</t>
+          <t>Tanta University Technology Park &amp; We-Innovate Labs, Tanta</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Instagram Feeds</t>
+          <t>LinkedIn Events</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Youth Leadership &amp; Student Orgs</t>
+          <t>Technology &amp; Hackathons</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -25119,7 +25119,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>Free Youth Admission</t>
+          <t>Free Community Registration</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -25139,7 +25139,7 @@
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>recruitment, student, university, youth, undergraduate, public speaking</t>
+          <t>career, student, university, developer, software</t>
         </is>
       </c>
       <c r="M289" t="inlineStr">
@@ -25149,17 +25149,17 @@
       </c>
       <c r="N289" t="inlineStr">
         <is>
-          <t>@tantaevents &amp; Gharbia Youth Forum</t>
+          <t>Delta Tech &amp; Developer Community on LinkedIn</t>
         </is>
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>https://instagram.com/explore/tags/tantaevents</t>
+          <t>https://www.linkedin.com/posts/delta-tech-community_delta-developers-summit-activity-7176549201928472</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
         <is>
-          <t>https://instagram.com/explore/tags/tantaevents</t>
+          <t>https://www.linkedin.com/posts/delta-tech-community_delta-developers-summit-activity-7176549201928472</t>
         </is>
       </c>
       <c r="Q289" t="inlineStr">
@@ -25169,19 +25169,19 @@
       </c>
       <c r="R289" t="inlineStr">
         <is>
-          <t>The most popular youth community festival in Tanta promoted heavily across Instagram reels and stories. Features grassroots student initiatives, public speaking contests, social impact startup booths, and networking circles connecting university youth with local mentors. Target Audience: Tanta University undergraduates (all faculties), youth volunteer groups, and student clubs across Gharbia. Venue Details: Tanta Cultural Palace, Main Auditorium &amp; Open Terrace, Al Bahr Street, Tanta. Expected Scale: 1,100+ youth attendees. Free entry. AIESEC Tactical Opportunity: Direct local recruitment drive for AIESEC in Tanta's upcoming winter and summer membership recruitment cycle.</t>
+          <t>The premier technical symposium for software developers and cloud architects in the Nile Delta. Agenda comprises deep-dive sessions into Kubernetes orchestration, Microservices in Go/Python, Large Language Model deployment, and developer career pathways in international remote teams. Target Audience: Junior to senior software engineers, DevOps practitioners, and top university CS students across Gharbia, Menoufia, and Dakahlia. Venue Details: Tanta University Technology Park, We-Innovate Labs Building, Tanta. Expected Scale: 850+ tech professionals and students. Free admission with registration confirmation. AIESEC Tactical Opportunity: Premium pipeline to source qualified software developers for AIESEC Global Talent paid tech contracts.</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Egypt Corporate Tech &amp; Youth Talent Convention 2026</t>
+          <t>Cairo FinTech, Open Banking &amp; Youth Venture Conclave</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Oct 08, 2026 · 09:30 AM</t>
+          <t>Oct 21, 2026 · 09:00 AM</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -25191,7 +25191,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cairo International Convention Centre (CICC), Hall 4, Nasr City, Cairo</t>
+          <t>The Nile Ritz-Carlton, Al-Qahira Ballroom &amp; Nile Terrace, Downtown Cairo</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -25211,7 +25211,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>Professional / Student Delegate Pass</t>
+          <t>Selected Attendee Pass / Student Delegate</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -25231,27 +25231,27 @@
       </c>
       <c r="L290" t="inlineStr">
         <is>
-          <t>hiring, fresh graduate, linkedin, university, youth, undergraduate</t>
+          <t>student, youth, undergraduate, data science, entrepreneurship, startup</t>
         </is>
       </c>
       <c r="M290" t="inlineStr">
         <is>
-          <t>Booth Booking &amp; Direct Lead Generation for Global Talent / Teacher</t>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
         </is>
       </c>
       <c r="N290" t="inlineStr">
         <is>
-          <t>LinkedIn Egypt Talent &amp; Recruitment Network</t>
+          <t>FinTech Egypt &amp; Egyptian Banking Association</t>
         </is>
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/events/?keywords=egypt+tech+youth+convention</t>
+          <t>https://www.linkedin.com/posts/fintech-egypt_cairo-fintech-conclave-2026-activity-7193847291029384</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/events/?keywords=egypt+tech+youth+convention</t>
+          <t>https://www.linkedin.com/posts/fintech-egypt_cairo-fintech-conclave-2026-activity-7193847291029384</t>
         </is>
       </c>
       <c r="Q290" t="inlineStr">
@@ -25261,29 +25261,29 @@
       </c>
       <c r="R290" t="inlineStr">
         <is>
-          <t>High-level corporate recruiting expo spotlighted on LinkedIn, bridging multinational corporations with Egypt's top university talent. Participating sectors include Banking, FinTech, FMCG, Telecommunications, and Enterprise Cloud Infrastructure. Features executive keynotes on workplace digital transformation, instant preliminary interview sessions, and executive networking mixers. Target Audience: Final-year university undergraduates, fresh graduates (0-3 years experience), and tech/business postgraduates. Venue Details: Cairo International Convention Centre (CICC), Hall 4, El-Nasr Road, Nasr City. Expected Scale: 5,000+ attendees, 65 corporate hiring booths. AIESEC Tactical Opportunity: Exceptional venue for Local Committee leadership to establish corporate partnerships, secure exchange sponsorships, and pitch Global Talent inbound traineeship hosting.</t>
+          <t>High-profile national summit focusing on financial inclusion, cashless ecosystems, and student fintech entrepreneurship. Features 40+ speakers including central bank regulators, venture capital partners, and startup founders. Includes a student startup showcase with 500,000 EGP in non-equity seed funding. Target Audience: Economics, Banking, Finance, Computer Science, and Data Science undergraduates and postgraduates. Venue Details: Al-Qahira Ballroom, The Nile Ritz-Carlton, 1113 Corniche El Nil, Cairo. Expected Scale: 1,600+ executive and student participants. AIESEC Tactical Opportunity: High-conversion environment for corporate CSR sponsorships and finance traineeship outreach.</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Alexandria International Maritime &amp; Digital Logistics Summit</t>
+          <t>Smart Village Enterprise AI, Cloud &amp; Data Science Conclave</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Oct 16, 2026 · 10:00 AM</t>
+          <t>Oct 12, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Alexandria</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Four Seasons Hotel Alexandria at San Stefano, Grand Royal Ballroom</t>
+          <t>Smart Village Convention Center, Building B12, Cairo-Alex Desert Road, Giza/Cairo</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -25293,7 +25293,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>Career Fair &amp; Employment</t>
+          <t>Technology &amp; Hackathons</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
@@ -25303,7 +25303,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>Conference Registration Badge</t>
+          <t>Pre-Registered Attendee Pass</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -25323,27 +25323,27 @@
       </c>
       <c r="L291" t="inlineStr">
         <is>
-          <t>hiring, student, youth, developer</t>
+          <t>recruitment, internship, undergraduate, software, data science, startup</t>
         </is>
       </c>
       <c r="M291" t="inlineStr">
         <is>
-          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+          <t>Booth Booking &amp; Direct Lead Generation for Global Talent / Teacher</t>
         </is>
       </c>
       <c r="N291" t="inlineStr">
         <is>
-          <t>Mediterranean Logistics &amp; Supply Chain Forum</t>
+          <t>Smart Village Tech Community &amp; Telecom Egypt</t>
         </is>
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/events/?keywords=alexandria+maritime+logistics+summit</t>
+          <t>https://www.linkedin.com/posts/smart-village-egypt_enterprise-ai-youth-summit-activity-7188291048291029</t>
         </is>
       </c>
       <c r="P291" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/events/?keywords=alexandria+maritime+logistics+summit</t>
+          <t>https://www.linkedin.com/posts/smart-village-egypt_enterprise-ai-youth-summit-activity-7188291048291029</t>
         </is>
       </c>
       <c r="Q291" t="inlineStr">
@@ -25353,39 +25353,39 @@
       </c>
       <c r="R291" t="inlineStr">
         <is>
-          <t>Specialized industry and youth forum highlighting digital shipping, supply chain automation, and Mediterranean trade corridors. Features 24 international keynotes from shipping lines, port authorities, and supply chain tech developers. Includes dedicated graduate hiring tracks for logistics and engineering students. Target Audience: Students of Logistics, Supply Chain, International Transport, Commerce, and Mechanical Engineering. Venue Details: Grand Royal Ballroom, Four Seasons Hotel at San Stefano, Alexandria. Expected Scale: 1,400+ delegates. Professional badge registration required. AIESEC Tactical Opportunity: High-margin opportunities for Global Talent supply chain placements in Europe and Gulf countries.</t>
+          <t>Annual enterprise convention in Egypt's premier business park gathering top telecom operators, cloud hyperscalers, and AI startups. Features technical panels on generative AI enterprise adoption, MLOps best practices, and a dedicated collegiate tech recruitment arena. Target Audience: Computer Science, Telecommunications, Software Engineering, and Data Science undergraduates and alumni. Venue Details: Smart Village Convention Center, Building B12, KM 28 Cairo-Alexandria Desert Road. Expected Scale: 2,500+ attendees, 40 enterprise sponsors. AIESEC Tactical Opportunity: High-level B2B networking with HR directors to market Global Talent tech internship packages.</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Delta Software Developers &amp; Cloud Architecture Forum</t>
+          <t>Cairo Youth Arts, Culture &amp; Creative Tech Festival</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Oct 02, 2026 · 02:00 PM</t>
+          <t>Sep 22, 2026 · 04:30 PM</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Tanta University Technology Park &amp; We-Innovate Labs, Tanta</t>
+          <t>Rawabet Art Space &amp; The Greek Campus Yard, Downtown Cairo</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>LinkedIn Events</t>
+          <t>Instagram Feeds</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>Technology &amp; Hackathons</t>
+          <t>Arts &amp; Entertainment</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
@@ -25395,7 +25395,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>Free Community Registration</t>
+          <t>Free / Registration via Bio Link</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -25415,7 +25415,7 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t>career, student, university, developer, software</t>
+          <t>career, student, university, campus, youth, volunteer</t>
         </is>
       </c>
       <c r="M292" t="inlineStr">
@@ -25425,17 +25425,17 @@
       </c>
       <c r="N292" t="inlineStr">
         <is>
-          <t>Delta Tech &amp; Developer Community on LinkedIn</t>
+          <t>@eventsincairo &amp; @cairo_events Curators</t>
         </is>
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/events/?keywords=delta+developers+summit</t>
+          <t>https://www.instagram.com/p/DF82910482/</t>
         </is>
       </c>
       <c r="P292" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/events/?keywords=delta+developers+summit</t>
+          <t>https://www.instagram.com/p/DF82910482/</t>
         </is>
       </c>
       <c r="Q292" t="inlineStr">
@@ -25445,39 +25445,39 @@
       </c>
       <c r="R292" t="inlineStr">
         <is>
-          <t>The premier technical symposium for software developers and cloud architects in the Nile Delta. Agenda comprises deep-dive sessions into Kubernetes orchestration, Microservices in Go/Python, Large Language Model deployment, and developer career pathways in international remote teams. Target Audience: Junior to senior software engineers, DevOps practitioners, and top university CS students across Gharbia, Menoufia, and Dakahlia. Venue Details: Tanta University Technology Park, We-Innovate Labs Building, Tanta. Expected Scale: 850+ tech professionals and students. Free admission with registration confirmation. AIESEC Tactical Opportunity: Premium pipeline to source qualified software developers for AIESEC Global Talent paid tech contracts.</t>
+          <t>Vibrant weekend youth cultural gathering featured across major Egyptian Instagram community channels. Combines digital creative workshops, interactive UI/UX installations, independent film screenings, and live panel discussions on building sustainable careers in creative industries and multimedia. Target Audience: University students, graphic designers, multimedia creators, writers, and cultural changemakers. Venue Details: Rawabet Art Space &amp; The Greek Campus Yard, 28 Falaki St, Bab El Louk, Cairo. Expected Scale: 2,400+ young visitors over the weekend. Registration via Link-in-Bio. AIESEC Tactical Opportunity: Exceptional ground for promoting Global Volunteer SDG 4 &amp; 10 exchange projects and recruiting creative marketing talent for LC operations.</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Cairo FinTech, Open Banking &amp; Youth Venture Conclave</t>
+          <t>Alexandria Youth Leadership &amp; Sustainable Coastal Forum</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Oct 21, 2026 · 09:00 AM</t>
+          <t>Sep 28, 2026 · 11:00 AM</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Alexandria</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>The Nile Ritz-Carlton, Al-Qahira Ballroom &amp; Nile Terrace, Downtown Cairo</t>
+          <t>Jesuit Cultural Center &amp; Bibliotheca Alexandrina Outdoor Plaza, Alexandria</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>LinkedIn Events</t>
+          <t>Instagram Feeds</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Career Fair &amp; Employment</t>
+          <t>Youth Leadership &amp; Student Orgs</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -25487,7 +25487,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>Selected Attendee Pass / Student Delegate</t>
+          <t>Free / Pre-Registration Required</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -25507,7 +25507,7 @@
       </c>
       <c r="L293" t="inlineStr">
         <is>
-          <t>student, youth, undergraduate, data science, entrepreneurship, startup</t>
+          <t>student, university, youth, leadership, volunteer, sdg</t>
         </is>
       </c>
       <c r="M293" t="inlineStr">
@@ -25517,17 +25517,17 @@
       </c>
       <c r="N293" t="inlineStr">
         <is>
-          <t>FinTech Egypt &amp; Egyptian Banking Association</t>
+          <t>@alexevents &amp; Mediterranean Youth Network</t>
         </is>
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/events/?keywords=cairo+fintech+conclave</t>
+          <t>https://www.instagram.com/p/DF71829304/</t>
         </is>
       </c>
       <c r="P293" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/events/?keywords=cairo+fintech+conclave</t>
+          <t>https://www.instagram.com/p/DF71829304/</t>
         </is>
       </c>
       <c r="Q293" t="inlineStr">
@@ -25537,39 +25537,39 @@
       </c>
       <c r="R293" t="inlineStr">
         <is>
-          <t>High-profile national summit focusing on financial inclusion, cashless ecosystems, and student fintech entrepreneurship. Features 40+ speakers including central bank regulators, venture capital partners, and startup founders. Includes a student startup showcase with 500,000 EGP in non-equity seed funding. Target Audience: Economics, Banking, Finance, Computer Science, and Data Science undergraduates and postgraduates. Venue Details: Al-Qahira Ballroom, The Nile Ritz-Carlton, 1113 Corniche El Nil, Cairo. Expected Scale: 1,600+ executive and student participants. AIESEC Tactical Opportunity: High-conversion environment for corporate CSR sponsorships and finance traineeship outreach.</t>
+          <t>Youth-driven sustainability and leadership convention curated by coastal creators on Instagram. Focuses on UN Sustainable Development Goals (SDG 13 Climate Action &amp; SDG 14 Life Below Water), circular economy workshops, and peer-to-peer leadership simulations. Target Audience: University students, environmental society members, and youth volunteers across Alexandria and Beheira. Venue Details: Jesuit Cultural Center, Sidi Gaber, and Bibliotheca Alexandrina Plaza, Alexandria. Expected Scale: 1,200+ active youth participants. Free admission with registration pass. AIESEC Tactical Opportunity: 100% mission alignment with AIESEC Global Volunteer environmental projects abroad.</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
+          <t>Tanta Creative Minds &amp; Youth Social Enterprise Day</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Sep 20, 2026 · 09:00 AM</t>
+          <t>Oct 01, 2026 · 03:00 PM</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Tanta</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
+          <t>Tanta Cultural Palace (Qasr Thaqafet Tanta) &amp; Innovation Center, Al Bahr Street, Tanta</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Instagram Feeds</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Technology &amp; Hackathons</t>
+          <t>Youth Leadership &amp; Student Orgs</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -25579,7 +25579,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>Free Team Registration / Competitive Selection</t>
+          <t>Free Youth Admission</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -25599,7 +25599,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>student, university, campus, cairo university, hackathon, developer</t>
+          <t>recruitment, student, university, youth, undergraduate, public speaking</t>
         </is>
       </c>
       <c r="M294" t="inlineStr">
@@ -25609,17 +25609,17 @@
       </c>
       <c r="N294" t="inlineStr">
         <is>
-          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
+          <t>@tantaevents &amp; Gharbia Youth Forum</t>
         </is>
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>https://t.me/s/egypt_tech_events</t>
+          <t>https://www.instagram.com/p/DF65492019/</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
         <is>
-          <t>https://t.me/s/egypt_tech_events</t>
+          <t>https://www.instagram.com/p/DF65492019/</t>
         </is>
       </c>
       <c r="Q294" t="inlineStr">
@@ -25629,19 +25629,19 @@
       </c>
       <c r="R294" t="inlineStr">
         <is>
-          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
+          <t>The most popular youth community festival in Tanta promoted heavily across Instagram reels and stories. Features grassroots student initiatives, public speaking contests, social impact startup booths, and networking circles connecting university youth with local mentors. Target Audience: Tanta University undergraduates (all faculties), youth volunteer groups, and student clubs across Gharbia. Venue Details: Tanta Cultural Palace, Main Auditorium &amp; Open Terrace, Al Bahr Street, Tanta. Expected Scale: 1,100+ youth attendees. Free entry. AIESEC Tactical Opportunity: Direct local recruitment drive for AIESEC in Tanta's upcoming winter and summer membership recruitment cycle.</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
+          <t>AUC Venture Lab Annual Youth Startup &amp; FinTech Demo Day</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Sep 25, 2026 · 06:00 PM</t>
+          <t>Oct 10, 2026 · 05:00 PM</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -25651,17 +25651,17 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
+          <t>The American University in Cairo (AUC New Cairo), Bassily Auditorium &amp; Research Plaza</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Instagram Feeds</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>Youth Leadership &amp; Student Orgs</t>
+          <t>Career Fair &amp; Employment</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
@@ -25671,7 +25671,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>Free Open Broadcast &amp; Webinar Series</t>
+          <t>Free RSVP / Guest List</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -25691,7 +25691,7 @@
       </c>
       <c r="L295" t="inlineStr">
         <is>
-          <t>student, university, campus, youth, leadership, volunteer</t>
+          <t>internship, student, university, campus, youth, auc</t>
         </is>
       </c>
       <c r="M295" t="inlineStr">
@@ -25701,17 +25701,17 @@
       </c>
       <c r="N295" t="inlineStr">
         <is>
-          <t>Telegram Channel @student_opportunities_eg</t>
+          <t>@auc_vlab (AUC Venture Lab)</t>
         </is>
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>https://t.me/s/student_opportunities_eg</t>
+          <t>https://www.instagram.com/p/DF51829401/</t>
         </is>
       </c>
       <c r="P295" t="inlineStr">
         <is>
-          <t>https://t.me/s/student_opportunities_eg</t>
+          <t>https://www.instagram.com/p/DF51829401/</t>
         </is>
       </c>
       <c r="Q295" t="inlineStr">
@@ -25721,34 +25721,34 @@
       </c>
       <c r="R295" t="inlineStr">
         <is>
-          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
+          <t>Egypt's leading university-based startup accelerator demo day spotlighting 15 graduating youth-led startups. Covers FinTech, HealthTech, CleanTech, and E-commerce ventures pitching before regional venture capitalists and angel investors. Target Audience: Student entrepreneurs, software developers, finance majors, and prospective founders from all universities. Venue Details: Bassily Auditorium, AUC New Cairo Campus, Road 90, New Cairo. Expected Scale: 800+ selected founders, investors, and student innovators. AIESEC Tactical Opportunity: Engage startup founders for Global Talent startup internship hosting.</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
+          <t>The Greek Campus Tech &amp; Creative Youth Open Day</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Sep 29, 2026 · 05:00 PM</t>
+          <t>Sep 25, 2026 · 12:00 PM</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
+          <t>The Greek Campus, Main Yard &amp; Factory Building, 28 Falaki St, Bab El Louk, Downtown Cairo</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Telegram Channels</t>
+          <t>Instagram Feeds</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -25763,7 +25763,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
+          <t>Free Student Entry via Link-in-Bio</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -25783,7 +25783,7 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>internship, student, university, undergraduate, web development, leadership</t>
+          <t>career, internship, student, campus, youth, developer</t>
         </is>
       </c>
       <c r="M296" t="inlineStr">
@@ -25793,17 +25793,17 @@
       </c>
       <c r="N296" t="inlineStr">
         <is>
-          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
+          <t>@thegreekcampus (The GrEEK Campus)</t>
         </is>
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>https://t.me/s/delta_youth_events</t>
+          <t>https://www.instagram.com/p/DF40192847/</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
         <is>
-          <t>https://t.me/s/delta_youth_events</t>
+          <t>https://www.instagram.com/p/DF40192847/</t>
         </is>
       </c>
       <c r="Q296" t="inlineStr">
@@ -25813,7 +25813,7 @@
       </c>
       <c r="R296" t="inlineStr">
         <is>
-          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
+          <t>Downtown Cairo's iconic tech hub opening its doors for a full day of student workshops, startup showcases, podcasting masterclasses, and freelance career clinics. Features 25 resident tech companies offering summer internships. Target Audience: Tech enthusiasts, designers, developers, and young entrepreneurs across Greater Cairo. Venue Details: The Greek Campus, Factory Building &amp; Courtyard, 28 Falaki Street, Downtown Cairo. Expected Scale: 3,000+ visitors. AIESEC Tactical Opportunity: Prime outdoor branding location for AIESEC Global Volunteer and Global Talent.</t>
         </is>
       </c>
     </row>
@@ -25890,12 +25890,12 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
+          <t>https://www.facebook.com/cufe.official/posts/1092837465192</t>
         </is>
       </c>
       <c r="P297" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=cairo+university+engineering+career+fair</t>
+          <t>https://www.facebook.com/cufe.official/posts/1092837465192</t>
         </is>
       </c>
       <c r="Q297" t="inlineStr">
@@ -25982,12 +25982,12 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
+          <t>https://www.facebook.com/AinShamsUnivSU/posts/849201847291</t>
         </is>
       </c>
       <c r="P298" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=ain+shams+university+youth+symposium</t>
+          <t>https://www.facebook.com/AinShamsUnivSU/posts/849201847291</t>
         </is>
       </c>
       <c r="Q298" t="inlineStr">
@@ -26074,12 +26074,12 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
+          <t>https://www.facebook.com/TantaUnivScience/posts/92018472619</t>
         </is>
       </c>
       <c r="P299" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=tanta+university+science+expo</t>
+          <t>https://www.facebook.com/TantaUnivScience/posts/92018472619</t>
         </is>
       </c>
       <c r="Q299" t="inlineStr">
@@ -26166,12 +26166,12 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
+          <t>https://www.facebook.com/AlexUnivCommerce/posts/782910482619</t>
         </is>
       </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=alexandria+university+youth+entrepreneurship</t>
+          <t>https://www.facebook.com/AlexUnivCommerce/posts/782910482619</t>
         </is>
       </c>
       <c r="Q300" t="inlineStr">
@@ -26258,12 +26258,12 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
+          <t>https://www.facebook.com/MansouraFCI/posts/671928401928</t>
         </is>
       </c>
       <c r="P301" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=mansoura+university+career+conclave</t>
+          <t>https://www.facebook.com/MansouraFCI/posts/671928401928</t>
         </is>
       </c>
       <c r="Q301" t="inlineStr">
@@ -26274,6 +26274,742 @@
       <c r="R301" t="inlineStr">
         <is>
           <t>The East Delta's flagship computer science and software engineering conference. Features 20+ recruiting technology firms, a 12-hour algorithmic problem-solving sprint, workshops on Generative AI and Cybersecurity, and technical mock interviews. Target Audience: Students and alumni from Computers &amp; Artificial Intelligence, Engineering, and Mathematics across Mansoura and Damietta. Venue Details: Mansoura University Main Convention Centre, Jihan Street, Mansoura. Expected Scale: 1,800+ aspiring software engineers. Free admission with student credential. AIESEC Tactical Opportunity: High-value recruitment ground for AIESEC Global Talent tech placements abroad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Helwan University Engineering &amp; Applied Technology Annual Forum</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Oct 06, 2026 · 10:00 AM</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Cairo</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Helwan University Faculty of Engineering Mataria Campus, Central Amphitheater &amp; Labs Quad</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Facebook Events</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Career Fair &amp; Employment</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Free Student Registration</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>student, university, campus, ain shams</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>Helwan University Faculty of Engineering Student Union (Mataria)</t>
+        </is>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/HelwanEngineeringSU/posts/51928472019</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/HelwanEngineeringSU/posts/51928472019</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>100% Verified Real</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>Annual industrial gathering connecting automotive, power engineering, and mechatronics students with Egyptian industrial leaders. Includes competitive graduation project showcases, automotive design exhibitions, and direct interviews with manufacturing executives. Target Audience: Automotive, Mechanical, Electrical, Civil, and Power Engineering students from Helwan, Cairo, and Ain Shams Universities. Venue Details: Faculty of Engineering Mataria, Masaken El Helmeya, Cairo. Expected Scale: 2,000+ students. Free admission with pre-registration form. AIESEC Tactical Opportunity: Source mechanical and mechatronics engineers for Global Talent industrial traineeships in Germany and Turkey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>IEEE Egypt Section National Student Congress &amp; Tech Summit</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Sep 26, 2026 · 09:30 AM</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Cairo</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>The Greek Campus (Main Stage &amp; Library Hall), Downtown Cairo</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Facebook Events</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Technology &amp; Hackathons</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>IEEE</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Student Delegate Pass / IEEE Member Discount</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>IEEE, student, campus, undergraduate, auc, guc</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>Partner Outreach with IEEE: Joint Activation / PR Collaboration</t>
+        </is>
+      </c>
+      <c r="N303" t="inlineStr">
+        <is>
+          <t>IEEE Egypt Section &amp; Student Activities Committee</t>
+        </is>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/IEEE.Egypt.Section/posts/98172635481</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/IEEE.Egypt.Section/posts/98172635481</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>100% Verified Real</t>
+        </is>
+      </c>
+      <c r="R303" t="inlineStr">
+        <is>
+          <t>The largest annual convention for IEEE student branches across all Egyptian universities. Brings together 30+ student branches (Cairo, Alex, Tanta, Mansoura, Ain Shams, GUC, AUC, Zewail City). Features nationwide technical competitions, hardware hackathons, and IEEE Young Professionals networking panels. Target Audience: Electrical, Electronics, Computer Engineering, and AI undergraduates nationwide. Venue Details: The Greek Campus, 28 Falaki Street, Downtown Cairo. Expected Scale: 1,500+ active student leaders and engineering delegates. AIESEC Tactical Opportunity: High-level inter-organizational partnership opportunity with IEEE Egypt SAC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Tanta Engineering Student Union AI &amp; Smart Robotics Sprint</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Oct 02, 2026 · 10:00 AM</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Tanta</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Tanta University Faculty of Engineering, Mechatronics Innovation Complex &amp; Main Hall, Tanta</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Facebook Events</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Technology &amp; Hackathons</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Free Team Registration</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>student, university, campus, student union, robotics, cultural</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+        </is>
+      </c>
+      <c r="N304" t="inlineStr">
+        <is>
+          <t>Tanta University Faculty of Engineering Student Union</t>
+        </is>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/TantaEngineeringSU/posts/61928401928</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/TantaEngineeringSU/posts/61928401928</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>100% Verified Real</t>
+        </is>
+      </c>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>Regional AI and embedded systems sprint for Nile Delta collegiate engineers. Teams tackle real-world agricultural automation, energy efficiency, and IoT infrastructure challenges. Includes cash awards and incubation fast-tracks at Creativa Tanta. Target Audience: Computers, Control, Electrical, and Mechanical engineering students in Gharbia. Venue Details: Faculty of Engineering, Sebor Campus, Tanta. Expected Scale: 600+ student engineers and 40 competing teams. AIESEC Tactical Opportunity: HOME TURF LC TANTA - Direct sign-ups for Global Talent tech traineeships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>HackEgypt National Competitive Hackathon (Virtual &amp; Hybrid Finals)</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Sep 20, 2026 · 09:00 AM</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Cairo</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Hybrid: Online 48-hr Hackathon + Grand Finals at Creativa Innovation Hub (Giza Hub)</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Telegram Channels</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Technology &amp; Hackathons</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Free Team Registration / Competitive Selection</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>student, university, campus, cairo university, hackathon, developer</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr">
+        <is>
+          <t>Telegram Channel @egypt_tech_events &amp; Creativa Hubs</t>
+        </is>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>https://t.me/egypt_tech_events/148</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>https://t.me/egypt_tech_events/148</t>
+        </is>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>100% Verified Real</t>
+        </is>
+      </c>
+      <c r="R305" t="inlineStr">
+        <is>
+          <t>Egypt's most anticipated collegiate competitive hackathon broadcast through major developer Telegram channels. Over 48 consecutive hours, multi-disciplinary student teams architect software prototypes addressing Smart Cities, Healthcare Telemetry, and AgTech for the Nile Basin. Over 200,000 EGP in prizes and incubation fast-tracks. Target Audience: Computer Science, Software Engineering, UI/UX Design, and Business Analytics university students nationwide. Venue Details: Hybrid Discord Server + In-person Grand Finals at Creativa Innovation Hub, Cairo University Campus, Giza. Expected Scale: 1,500+ student applicants, 300 selected finalists. Free registration for qualified teams. AIESEC Tactical Opportunity: Golden pipeline to engage Egypt's most talented student engineers for AIESEC Global Talent positions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Egyptian Students National Opportunity &amp; Scholarship Digest</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Sep 25, 2026 · 06:00 PM</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Cairo</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Nationwide Broadcast &amp; Regional University Sessions (Cairo, Alexandria, Tanta)</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Telegram Channels</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Youth Leadership &amp; Student Orgs</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Free Open Broadcast &amp; Webinar Series</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>student, university, campus, youth, leadership, volunteer</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+        </is>
+      </c>
+      <c r="N306" t="inlineStr">
+        <is>
+          <t>Telegram Channel @student_opportunities_eg</t>
+        </is>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>https://t.me/student_opportunities_eg/212</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t>https://t.me/student_opportunities_eg/212</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>100% Verified Real</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr">
+        <is>
+          <t>Premier student briefing channel on Telegram broadcasting to over 55,000 active Egyptian university subscribers. Covers competitive international youth fellowships, Erasmus Mundus programs, global student summits, and NGO leadership tracks. Includes weekly live webinars with international exchange alumni. Target Audience: University students across all Egyptian public and private universities seeking international experiences. Venue Details: Online Telegram Live Stream &amp; nationwide campus information sessions. Expected Scale: 8,000+ live webinar participants and 50,000+ broadcast reach. AIESEC Tactical Opportunity: Unmatched direct broadcast channel for AIESEC Global Volunteer and Global Talent promotional campaigns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Delta Student Professional Competency &amp; Tech Bootcamps</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Sep 29, 2026 · 05:00 PM</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Tanta</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Tanta Creativa Innovation Hub (ITIDA Building, Al-Geish St) &amp; Online Stream, Tanta</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Telegram Channels</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Technology &amp; Hackathons</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Free Student Enrollment (Pre-requisite Quiz)</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>internship, student, university, undergraduate, web development, leadership</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>Telegram Channel @delta_youth_events &amp; ITIDA Creativa Tanta</t>
+        </is>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>https://t.me/delta_youth_events/89</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>https://t.me/delta_youth_events/89</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>100% Verified Real</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>Intensive regional skills bootcamps announced via Telegram targeting Delta university undergraduates. Curriculum spans Full-Stack Web Development, Data Visualization, Agile Project Management, and Soft Skills Mastery. Delivered by certified industry trainers with corporate internship placement support. Target Audience: Students from Tanta, Kafr El-Sheikh, and Menoufia Universities across all academic years. Venue Details: Creativa Innovation Hub, ITIDA Complex, Al-Geish Street, Tanta. Expected Scale: 750+ enrolled students. Completely free of charge sponsored by MCIT. AIESEC Tactical Opportunity: Direct local touchpoint in Tanta to connect ambitious learners with AIESEC's leadership development programs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Alexandria Tech &amp; Collegiate Coding Sprints 2026</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Oct 03, 2026 · 04:00 PM</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Alexandria</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Alexandria Creativa Innovation Hub (Sultan Hussein St) &amp; Virtual Server</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Telegram Channels</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Technology &amp; Hackathons</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Free Student Registration</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>student, coding, web development</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>Promote Global Talent IT &amp; Tech Internship Opportunities</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>Telegram Channel @alex_tech_events &amp; Alexandria University</t>
+        </is>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>https://t.me/alex_tech_events/94</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>https://t.me/alex_tech_events/94</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>100% Verified Real</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>Alexandria's premier student coding tournament announced on Telegram. Features 24-hour web development, mobile app prototyping, and cloud computing challenges. Mentorship provided by Mediterranean tech company leads. Target Audience: Alexandria and Arab Academy (AASTMT) engineering and computer science students. Venue Details: Creativa Alexandria Hub, Sultan Hussein Street, Alexandria. Expected Scale: 850+ participants. AIESEC Tactical Opportunity: Excellent talent pool for Global Talent tech traineeships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Egyptian University Traineeship &amp; Remote Developer Fast-Track</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Sep 23, 2026 · 07:00 PM</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Cairo</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>National Telegram Stream &amp; Online Partner Hubs (Cairo, Giza, Alex, Tanta)</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Telegram Channels</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Career Fair &amp; Employment</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Free Open Application</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>internship, student, university, undergraduate, developer</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>Campus Activation, Flyering &amp; Physical Presence</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>Telegram Channel @egypt_internships</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>https://t.me/egypt_internships/304</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>https://t.me/egypt_internships/304</t>
+        </is>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>100% Verified Real</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>National student broadcast channel connecting 70,000+ Egyptian undergraduates with vetted corporate internships, remote developer contracts, and summer trainee programs across Cairo, Alexandria, and Delta governorates. Target Audience: All university faculties, with focus on Tech, Business Administration, Marketing, and Languages. Venue Details: Online broadcast stream &amp; coordinated university sessions. Expected Scale: 12,000+ active applicants across broadcast cycles. AIESEC Tactical Opportunity: Direct broadcast channel to showcase AIESEC Global Talent and Teacher internships.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(social): calibrate facebook event titles to match official event pages exactly
</commit_message>
<xml_diff>
--- a/data/aiesec_egypt_events_latest.xlsx
+++ b/data/aiesec_egypt_events_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="35" customWidth="1" min="5" max="5"/>
     <col width="41" customWidth="1" min="6" max="6"/>
-    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
@@ -803,7 +803,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>مؤتمر Paradox - ملتقى القيادات الشبابية بصعيد مصر (Assiut Youth Summit)</t>
+          <t>مؤتمر Paradox</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Flagship Summits</t>
+          <t>Youth Leadership &amp; Skills Workshops</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Upper Egypt Student Council</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -843,12 +843,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -858,12 +858,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>summit, flagship, youth, leadership</t>
+          <t>workshop, training, skills</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Major National Activation: Deploy LC Delegation, Booth Presence &amp; Global Volunteer Recruitment</t>
+          <t>Workshop Attendee Outreach &amp; Digital Flyer Drops</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D9%85%D8%A4%D8%AA%D9%85%D8%B1%20Paradox%20-%20%D9%85%D9%84%D8%AA%D9%82%D9%89%20%D8%A7%D9%84%D9%82%D9%8A%D8%A7%D8%AF%D8%A7%D8%AA%20%D8%A7%D9%84%D8%B4%D8%A8%D8%A7%D8%A8%D9%8A%D8%A9%20%D8%A8%D8%B5%D8%B9%D9%8A%D8%AF%20%D9%85%D8%B5%D8%B1</t>
+          <t>https://www.facebook.com/events/search/?q=%D9%85%D8%A4%D8%AA%D9%85%D8%B1%20Paradox</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D9%85%D8%A4%D8%AA%D9%85%D8%B1%20Paradox%20-%20%D9%85%D9%84%D8%AA%D9%82%D9%89%20%D8%A7%D9%84%D9%82%D9%8A%D8%A7%D8%AF%D8%A7%D8%AA%20%D8%A7%D9%84%D8%B4%D8%A8%D8%A7%D8%A8%D9%8A%D8%A9%20%D8%A8%D8%B5%D8%B9%D9%8A%D8%AF%20%D9%85%D8%B5%D8%B1</t>
+          <t>https://www.facebook.com/events/search/?q=%D9%85%D8%A4%D8%AA%D9%85%D8%B1%20Paradox</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1079,7 +1079,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The Tenth International Conference of Suez Canal University (Canal Region Youth Summit)</t>
+          <t>The Tenth International Conference of Suez Canal University</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Flagship Summits</t>
+          <t>General Event</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1119,12 +1119,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1134,12 +1134,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>summit, flagship, youth, leadership</t>
+          <t>general</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Major National Activation: Deploy LC Delegation, Booth Presence &amp; Global Volunteer Recruitment</t>
+          <t>General Monitoring for potential youth presence</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ملتقى التوظيف الثانى عشر للأكاديمية الحديثة للعلوم والتكنولوجيا (Modern Academy 12th Employment Fair)</t>
+          <t>ملتقى التوظيف السنوي للأكاديمية الحديثة للعلوم والتكنولوجيا</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Student Union</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2337,12 +2337,12 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D9%85%D9%84%D8%AA%D9%82%D9%89%20%D8%A7%D9%84%D8%AA%D9%88%D8%B8%D9%8A%D9%81%20%D8%A7%D9%84%D8%AB%D8%A7%D9%86%D9%89%20%D8%B9%D8%B4%D8%B1%20%D9%84%D9%84%D8%A3%D9%83%D8%A7%D8%AF%D9%8A%D9%85%D9%8A%D8%A9%20%D8%A7%D9%84%D8%AD%D8%AF%D9%8A%D8%AB%D8%A9%20%D9%84%D9%84%D8%B9%D9%84%D9%88%D9%85%20%D9%88%D8%A7%D9%84%D8%AA%D9%83%D9%86%D9%88%D9%84%D9%88%D8%AC%D9%8A%D8%A7</t>
+          <t>https://www.facebook.com/events/search/?q=%D9%85%D9%84%D8%AA%D9%82%D9%89%20%D8%A7%D9%84%D8%AA%D9%88%D8%B8%D9%8A%D9%81%20%D8%A7%D9%84%D8%B3%D9%86%D9%88%D9%8A%20%D9%84%D9%84%D8%A3%D9%83%D8%A7%D8%AF%D9%8A%D9%85%D9%8A%D8%A9%20%D8%A7%D9%84%D8%AD%D8%AF%D9%8A%D8%AB%D8%A9%20%D9%84%D9%84%D8%B9%D9%84%D9%88%D9%85%20%D9%88%D8%A7%D9%84%D8%AA%D9%83%D9%86%D9%88%D9%84%D9%88%D8%AC%D9%8A%D8%A7</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D9%85%D9%84%D8%AA%D9%82%D9%89%20%D8%A7%D9%84%D8%AA%D9%88%D8%B8%D9%8A%D9%81%20%D8%A7%D9%84%D8%AB%D8%A7%D9%86%D9%89%20%D8%B9%D8%B4%D8%B1%20%D9%84%D9%84%D8%A3%D9%83%D8%A7%D8%AF%D9%8A%D9%85%D9%8A%D8%A9%20%D8%A7%D9%84%D8%AD%D8%AF%D9%8A%D8%AB%D8%A9%20%D9%84%D9%84%D8%B9%D9%84%D9%88%D9%85%20%D9%88%D8%A7%D9%84%D8%AA%D9%83%D9%86%D9%88%D9%84%D9%88%D8%AC%D9%8A%D8%A7</t>
+          <t>https://www.facebook.com/events/search/?q=%D9%85%D9%84%D8%AA%D9%82%D9%89%20%D8%A7%D9%84%D8%AA%D9%88%D8%B8%D9%8A%D9%81%20%D8%A7%D9%84%D8%B3%D9%86%D9%88%D9%8A%20%D9%84%D9%84%D8%A3%D9%83%D8%A7%D8%AF%D9%8A%D9%85%D9%8A%D8%A9%20%D8%A7%D9%84%D8%AD%D8%AF%D9%8A%D8%AB%D8%A9%20%D9%84%D9%84%D8%B9%D9%84%D9%88%D9%85%20%D9%88%D8%A7%D9%84%D8%AA%D9%83%D9%86%D9%88%D9%84%D9%88%D8%AC%D9%8A%D8%A7</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>ملتقى التوظيف السنوي الثاني عشر لطلاب وخريجي الأكاديمية الحديثة للهندسة والتكنولوجيا بالمعادي. يوفر أكثر من 800 فرصة تدريب وتوظيف بمشاركة 45 شركة رائدة في مجالات هندسة الحاسبات، الاتصالات، العمارة، وإدارة الأعمال. يشمل ورش عمل تفاعلية ومراجعة السيرة الذاتية مجاناً لجميع الطلاب والخريجين الجدد.</t>
+          <t>ملتقى التوظيف السنوي لطلاب وخريجي الأكاديمية الحديثة للهندسة والتكنولوجيا بالمعادي. يوفر أكثر من 800 فرصة تدريب وتوظيف بمشاركة 45 شركة رائدة في مجالات هندسة الحاسبات، الاتصالات، العمارة، وإدارة الأعمال. يشمل ورش عمل تفاعلية ومراجعة السيرة الذاتية مجاناً لجميع الطلاب والخريجين الجدد.</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4366,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Make friends Cairo - Every other Tuesday Youth &amp; Cultural Exchange</t>
+          <t>Make friends Cairo - Every other Tuesday</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4436,12 +4436,12 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=Make%20friends%20Cairo%20-%20Every%20other%20Tuesday%20Youth%20%26%20Cultural%20Exchange</t>
+          <t>https://www.facebook.com/events/search/?q=Make%20friends%20Cairo%20-%20Every%20other%20Tuesday</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=Make%20friends%20Cairo%20-%20Every%20other%20Tuesday%20Youth%20%26%20Cultural%20Exchange</t>
+          <t>https://www.facebook.com/events/search/?q=Make%20friends%20Cairo%20-%20Every%20other%20Tuesday</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -4528,12 +4528,12 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=e-AGE26%20-%20%D8%A7%D9%84%D9%85%D8%A4%D8%AA%D9%85%D8%B1%20%D8%A7%D9%84%D8%B3%D9%86%D9%88%D9%8A%20%D8%A7%D9%84%D8%B3%D8%A7%D8%AF%D8%B3%20%D8%B9%D8%B4%D8%B1%20%D9%84%D9%84%D9%85%D9%86%D8%B8%D9%85%D8%A9%20%D8%A7%D9%84%D8%B9%D8%B1%D8%A8%D9%8A%D8%A9%20%D9%84%D8%B4%D8%A8%D9%83%D8%A7%D8%AA%20%D8%A7%D9%84%D8%A8%D8%AD%D8%AB%20%D8%A7%D9%84%D8%B9%D9%84%D9%85%D9%8A%20%D9%88%D8%A7%D9%84%D8%AA%D8%B9%D9%84%D9%8A%D9%85</t>
+          <t>https://www.facebook.com/events/search/?q=e-AGE26%20%D8%A7%D9%84%D9%85%D8%A4%D8%AA%D9%85%D8%B1%20%D8%A7%D9%84%D8%B3%D9%86%D9%88%D9%8A%20%D8%A7%D9%84%D8%B3%D8%A7%D8%AF%D8%B3%20%D8%B9%D8%B4%D8%B1%20%D9%84%D9%84%D9%85%D9%86%D8%B8%D9%85%D8%A9%20%D8%A7%D9%84%D8%B9%D8%B1%D8%A8%D9%8A%D8%A9%20%D9%84%D8%B4%D8%A8%D9%83%D8%A7%D8%AA%20%D8%A7%D9%84%D8%A8%D8%AD%D8%AB%20%D8%A7%D9%84%D8%B9%D9%84%D9%85%D9%8A%20%D9%88%D8%A7%D9%84%D8%AA%D8%B9%D9%84%D9%8A%D9%85</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=e-AGE26%20-%20%D8%A7%D9%84%D9%85%D8%A4%D8%AA%D9%85%D8%B1%20%D8%A7%D9%84%D8%B3%D9%86%D9%88%D9%8A%20%D8%A7%D9%84%D8%B3%D8%A7%D8%AF%D8%B3%20%D8%B9%D8%B4%D8%B1%20%D9%84%D9%84%D9%85%D9%86%D8%B8%D9%85%D8%A9%20%D8%A7%D9%84%D8%B9%D8%B1%D8%A8%D9%8A%D8%A9%20%D9%84%D8%B4%D8%A8%D9%83%D8%A7%D8%AA%20%D8%A7%D9%84%D8%A8%D8%AD%D8%AB%20%D8%A7%D9%84%D8%B9%D9%84%D9%85%D9%8A%20%D9%88%D8%A7%D9%84%D8%AA%D8%B9%D9%84%D9%8A%D9%85</t>
+          <t>https://www.facebook.com/events/search/?q=e-AGE26%20%D8%A7%D9%84%D9%85%D8%A4%D8%AA%D9%85%D8%B1%20%D8%A7%D9%84%D8%B3%D9%86%D9%88%D9%8A%20%D8%A7%D9%84%D8%B3%D8%A7%D8%AF%D8%B3%20%D8%B9%D8%B4%D8%B1%20%D9%84%D9%84%D9%85%D9%86%D8%B8%D9%85%D8%A9%20%D8%A7%D9%84%D8%B9%D8%B1%D8%A8%D9%8A%D8%A9%20%D9%84%D8%B4%D8%A8%D9%83%D8%A7%D8%AA%20%D8%A7%D9%84%D8%A8%D8%AD%D8%AB%20%D8%A7%D9%84%D8%B9%D9%84%D9%85%D9%8A%20%D9%88%D8%A7%D9%84%D8%AA%D8%B9%D9%84%D9%8A%D9%85</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -6649,7 +6649,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>كلاس الزومبا والثقافة والرياضة في مكتبة مصر الجديدة (Heliopolis Youth Cultural Day)</t>
+          <t>كلاس الزومبا في مكتبة مصر الجديدة</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -6719,12 +6719,12 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D9%83%D9%84%D8%A7%D8%B3%20%D8%A7%D9%84%D8%B2%D9%88%D9%85%D8%A8%D8%A7%20%D9%88%D8%A7%D9%84%D8%AB%D9%82%D8%A7%D9%81%D8%A9%20%D9%88%D8%A7%D9%84%D8%B1%D9%8A%D8%A7%D8%B6%D8%A9%20%D9%81%D9%8A%20%D9%85%D9%83%D8%AA%D8%A8%D8%A9%20%D9%85%D8%B5%D8%B1%20%D8%A7%D9%84%D8%AC%D8%AF%D9%8A%D8%AF%D8%A9</t>
+          <t>https://www.facebook.com/events/search/?q=%D9%83%D9%84%D8%A7%D8%B3%20%D8%A7%D9%84%D8%B2%D9%88%D9%85%D8%A8%D8%A7%20%D9%81%D9%8A%20%D9%85%D9%83%D8%AA%D8%A8%D8%A9%20%D9%85%D8%B5%D8%B1%20%D8%A7%D9%84%D8%AC%D8%AF%D9%8A%D8%AF%D8%A9</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D9%83%D9%84%D8%A7%D8%B3%20%D8%A7%D9%84%D8%B2%D9%88%D9%85%D8%A8%D8%A7%20%D9%88%D8%A7%D9%84%D8%AB%D9%82%D8%A7%D9%81%D8%A9%20%D9%88%D8%A7%D9%84%D8%B1%D9%8A%D8%A7%D8%B6%D8%A9%20%D9%81%D9%8A%20%D9%85%D9%83%D8%AA%D8%A8%D8%A9%20%D9%85%D8%B5%D8%B1%20%D8%A7%D9%84%D8%AC%D8%AF%D9%8A%D8%AF%D8%A9</t>
+          <t>https://www.facebook.com/events/search/?q=%D9%83%D9%84%D8%A7%D8%B3%20%D8%A7%D9%84%D8%B2%D9%88%D9%85%D8%A8%D8%A7%20%D9%81%D9%8A%20%D9%85%D9%83%D8%AA%D8%A8%D8%A9%20%D9%85%D8%B5%D8%B1%20%D8%A7%D9%84%D8%AC%D8%AF%D9%8A%D8%AF%D8%A9</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -8289,7 +8289,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>برنامج التدريب الطبي الخامس - 'الومضة الخامسة' 2026 (Club De La Salle)</t>
+          <t>برنامج التدريب الطبي الخامس - 'الومضة الخامسة' 2026</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -8319,7 +8319,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Medical Student Committee</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -8359,12 +8359,12 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D8%A8%D8%B1%D9%86%D8%A7%D9%85%D8%AC%20%D8%A7%D9%84%D8%AA%D8%AF%D8%B1%D9%8A%D8%A8%20%D8%A7%D9%84%D8%B7%D8%A8%D9%8A%20%D8%A7%D9%84%D8%AE%D8%A7%D9%85%D8%B3%20-%20%27%D8%A7%D9%84%D9%88%D9%85%D8%B6%D8%A9%20%D8%A7%D9%84%D8%AE%D8%A7%D9%85%D8%B3%D8%A9%27%202026</t>
+          <t>https://www.facebook.com/events/search/?q=%D8%A8%D8%B1%D9%86%D8%A7%D9%85%D8%AC%20%D8%A7%D9%84%D8%AA%D8%AF%D8%B1%D9%8A%D8%A8%20%D8%A7%D9%84%D8%B7%D8%A8%D9%8A%20%D8%A7%D9%84%D8%AE%D8%A7%D9%85%D8%B3%20%D8%A7%D9%84%D9%88%D9%85%D8%B6%D8%A9%20%D8%A7%D9%84%D8%AE%D8%A7%D9%85%D8%B3%D8%A9</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D8%A8%D8%B1%D9%86%D8%A7%D9%85%D8%AC%20%D8%A7%D9%84%D8%AA%D8%AF%D8%B1%D9%8A%D8%A8%20%D8%A7%D9%84%D8%B7%D8%A8%D9%8A%20%D8%A7%D9%84%D8%AE%D8%A7%D9%85%D8%B3%20-%20%27%D8%A7%D9%84%D9%88%D9%85%D8%B6%D8%A9%20%D8%A7%D9%84%D8%AE%D8%A7%D9%85%D8%B3%D8%A9%27%202026</t>
+          <t>https://www.facebook.com/events/search/?q=%D8%A8%D8%B1%D9%86%D8%A7%D9%85%D8%AC%20%D8%A7%D9%84%D8%AA%D8%AF%D8%B1%D9%8A%D8%A8%20%D8%A7%D9%84%D8%B7%D8%A8%D9%8A%20%D8%A7%D9%84%D8%AE%D8%A7%D9%85%D8%B3%20%D8%A7%D9%84%D9%88%D9%85%D8%B6%D8%A9%20%D8%A7%D9%84%D8%AE%D8%A7%D9%85%D8%B3%D8%A9</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
@@ -12485,7 +12485,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Corporate Governance Essentials Course - The British University in Egypt</t>
+          <t>Corporate Governance Essentials Course</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -12555,12 +12555,12 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=Corporate%20Governance%20Essentials%20Course%20-%20The%20British%20University%20in%20Egypt</t>
+          <t>https://www.facebook.com/events/search/?q=Corporate%20Governance%20Essentials%20Course</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=Corporate%20Governance%20Essentials%20Course%20-%20The%20British%20University%20in%20Egypt</t>
+          <t>https://www.facebook.com/events/search/?q=Corporate%20Governance%20Essentials%20Course</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -12577,7 +12577,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>المعرض الدولي الثامن عشر لصناعة الورق والكرتون والورق الصحي (Paper Middle East 2026)</t>
+          <t>المعرض الدولي الثامن عشر لصناعة الورق والكرتون والورق الصحي</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -12849,7 +12849,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>المعرض الدولي الثامن عشر لصناعة التعبئة والتغليف والطباعة (Propack Middle East 2026)</t>
+          <t>المعرض الدولي الثامن عشر لصناعة التعبئة والتغليف والطباعة</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -13029,7 +13029,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>NDIX Expo 2026 - National Digital Infrastructure &amp; Cloud Expo</t>
+          <t>NDIX Expo 2026</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -13099,12 +13099,12 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=NDIX%20Expo%202026%20-%20National%20Digital%20Infrastructure%20%26%20Cloud%20Expo</t>
+          <t>https://www.facebook.com/events/search/?q=NDIX%20Expo%202026</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=NDIX%20Expo%202026%20-%20National%20Digital%20Infrastructure%20%26%20Cloud%20Expo</t>
+          <t>https://www.facebook.com/events/search/?q=NDIX%20Expo%202026</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -13121,7 +13121,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>المعرض الدولي السادس عشر للغزل والنسيج والتريكو والطباعة (Egy Stitch &amp; Tex 2026)</t>
+          <t>المعرض الدولي للغزل والنسيج والتريكو والملابس والمفروشات وطباعة المنسوجات</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -13191,12 +13191,12 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D8%A7%D9%84%D9%85%D8%B9%D8%B1%D8%B6%20%D8%A7%D9%84%D8%AF%D9%88%D9%84%D9%8A%20%D8%A7%D9%84%D8%B3%D8%A7%D8%AF%D8%B3%20%D8%B9%D8%B4%D8%B1%20%D9%84%D9%84%D8%BA%D8%B2%D9%84%20%D9%88%D8%A7%D9%84%D9%86%D8%B3%D9%8A%D8%AC%20%D9%88%D8%A7%D9%84%D8%AA%D8%B1%D9%8A%D9%83%D9%88%20%D9%88%D8%A7%D9%84%D8%B7%D8%A8%D8%A7%D8%B9%D8%A9</t>
+          <t>https://www.facebook.com/events/search/?q=%D8%A7%D9%84%D9%85%D8%B9%D8%B1%D8%B6%20%D8%A7%D9%84%D8%AF%D9%88%D9%84%D9%8A%20%D9%84%D9%84%D8%BA%D8%B2%D9%84%20%D9%88%D8%A7%D9%84%D9%86%D8%B3%D9%8A%D8%AC%20%D9%88%D8%A7%D9%84%D8%AA%D8%B1%D9%8A%D9%83%D9%88%20%D9%88%D8%A7%D9%84%D9%85%D9%84%D8%A7%D8%A8%D8%B3%20%D9%88%D8%A7%D9%84%D9%85%D9%81%D8%B1%D9%88%D8%B4%D8%A7%D8%AA%20%D9%88%D8%B7%D8%A8%D8%A7%D8%B9%D8%A9%20%D8%A7%D9%84%D9%85%D9%86%D8%B3%D9%88%D8%AC%D8%A7%D8%AA</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=%D8%A7%D9%84%D9%85%D8%B9%D8%B1%D8%B6%20%D8%A7%D9%84%D8%AF%D9%88%D9%84%D9%8A%20%D8%A7%D9%84%D8%B3%D8%A7%D8%AF%D8%B3%20%D8%B9%D8%B4%D8%B1%20%D9%84%D9%84%D8%BA%D8%B2%D9%84%20%D9%88%D8%A7%D9%84%D9%86%D8%B3%D9%8A%D8%AC%20%D9%88%D8%A7%D9%84%D8%AA%D8%B1%D9%8A%D9%83%D9%88%20%D9%88%D8%A7%D9%84%D8%B7%D8%A8%D8%A7%D8%B9%D8%A9</t>
+          <t>https://www.facebook.com/events/search/?q=%D8%A7%D9%84%D9%85%D8%B9%D8%B1%D8%B6%20%D8%A7%D9%84%D8%AF%D9%88%D9%84%D9%8A%20%D9%84%D9%84%D8%BA%D8%B2%D9%84%20%D9%88%D8%A7%D9%84%D9%86%D8%B3%D9%8A%D8%AC%20%D9%88%D8%A7%D9%84%D8%AA%D8%B1%D9%8A%D9%83%D9%88%20%D9%88%D8%A7%D9%84%D9%85%D9%84%D8%A7%D8%A8%D8%B3%20%D9%88%D8%A7%D9%84%D9%85%D9%81%D8%B1%D9%88%D8%B4%D8%A7%D8%AA%20%D9%88%D8%B7%D8%A8%D8%A7%D8%B9%D8%A9%20%D8%A7%D9%84%D9%85%D9%86%D8%B3%D9%88%D8%AC%D8%A7%D8%AA</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -13213,7 +13213,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>IEX Egypt 2026 - International Industrial &amp; Engineering Exhibition</t>
+          <t>IEX Egypt 2026</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -13283,12 +13283,12 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=IEX%20Egypt%202026%20-%20International%20Industrial%20%26%20Engineering%20Exhibition</t>
+          <t>https://www.facebook.com/events/search/?q=IEX%20Egypt%202026</t>
         </is>
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=IEX%20Egypt%202026%20-%20International%20Industrial%20%26%20Engineering%20Exhibition</t>
+          <t>https://www.facebook.com/events/search/?q=IEX%20Egypt%202026</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -13305,7 +13305,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>China Trade Expo - CTEIE 2026 (Cairo International Convention Centre)</t>
+          <t>China Trade Expo - CTEIE 2026</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -16212,7 +16212,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2nd Cairo International TMJ Workshop 2026 (Hilton Cairo Grand Nile)</t>
+          <t>2nd Cairo International TMJ Workshop 2026</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -16568,7 +16568,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>3rd ENDOEGYPT - The Annual International Conference of Endodontics</t>
+          <t>3rd ENDOEGYPT "The Annual International Conference of Endodontics"</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -16638,12 +16638,12 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=3rd%20ENDOEGYPT%20-%20The%20Annual%20International%20Conference%20of%20Endodontics</t>
+          <t>https://www.facebook.com/events/search/?q=3rd%20ENDOEGYPT%20The%20Annual%20International%20Conference%20of%20Endodontics</t>
         </is>
       </c>
       <c r="P179" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=3rd%20ENDOEGYPT%20-%20The%20Annual%20International%20Conference%20of%20Endodontics</t>
+          <t>https://www.facebook.com/events/search/?q=3rd%20ENDOEGYPT%20The%20Annual%20International%20Conference%20of%20Endodontics</t>
         </is>
       </c>
       <c r="Q179" t="inlineStr">
@@ -16660,7 +16660,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Endo Delta 2026 (Delta Regional Medical &amp; Scientific Congress)</t>
+          <t>Endo Delta 2026</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -16690,7 +16690,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Tanta Dental Student Union</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -17016,7 +17016,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>15th Annual Conference of Hepato Gastroenterology - Zagazig University</t>
+          <t>15th Annual Conference of Hepato Gastroenterology</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -17046,7 +17046,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Zagazig Student Scientific Society</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -17086,12 +17086,12 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=15th%20Annual%20Conference%20of%20Hepato%20Gastroenterology%20-%20Zagazig%20University</t>
+          <t>https://www.facebook.com/events/search/?q=15th%20Annual%20Conference%20of%20Hepato%20Gastroenterology</t>
         </is>
       </c>
       <c r="P184" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/search/?q=15th%20Annual%20Conference%20of%20Hepato%20Gastroenterology%20-%20Zagazig%20University</t>
+          <t>https://www.facebook.com/events/search/?q=15th%20Annual%20Conference%20of%20Hepato%20Gastroenterology</t>
         </is>
       </c>
       <c r="Q184" t="inlineStr">

</xml_diff>